<commit_message>
serach fixed & taps updated
</commit_message>
<xml_diff>
--- a/src/data/rozliv.xlsx
+++ b/src/data/rozliv.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="711">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="717">
   <si>
     <t>Наименование</t>
   </si>
@@ -665,6 +665,9 @@
     <t>Rakovar, РОЗЛИВ, Чехия</t>
   </si>
   <si>
+    <t>Red Button - Farout Faded Fantasy Super Grand Sale (Lager), РОЗЛИВ, Россия</t>
+  </si>
+  <si>
     <t>Red Button - Fondue fountain (Milk stout), РОЗЛИВ, Россия</t>
   </si>
   <si>
@@ -761,6 +764,9 @@
     <t>Saint Loony - NICE (Sour), РОЗЛИВ, Россия</t>
   </si>
   <si>
+    <t>Saint Loony - Strobe (Sour), РОЗЛИВ, Россия</t>
+  </si>
+  <si>
     <t>Saldens - Citra &amp; Galaxy Double IPA, РОЗЛИВ, Россия</t>
   </si>
   <si>
@@ -1577,6 +1583,9 @@
     <t>вынос_Plan B - Ковбой Мальборо (IPA), РОЗЛИВ, Россия</t>
   </si>
   <si>
+    <t>вынос_Red Button - Farout Faded Fantasy Super Grand Sale (Lager), РОЗЛИВ, Россия</t>
+  </si>
+  <si>
     <t>вынос_Red Button - Fondue fountain (Milk stout), РОЗЛИВ, Россия</t>
   </si>
   <si>
@@ -1622,6 +1631,9 @@
     <t>вынос_Saint Loony - NICE (Sour), РОЗЛИВ, Россия</t>
   </si>
   <si>
+    <t>вынос_Saint Loony - Strobe (Sour), РОЗЛИВ, Россия</t>
+  </si>
+  <si>
     <t>вынос_Saliwa - Death by a 1000 Cats (Triple IPA), РОЗЛИВ, Россия</t>
   </si>
   <si>
@@ -1931,6 +1943,9 @@
     <t>вынос_Одна тонна - Sunday Draft: Enigma + Idaho 7 (NE Pale Ale), РОЗЛИВ, Россия</t>
   </si>
   <si>
+    <t>вынос_Одна тонна - Коник (Kolsch), РОЗЛИВ, Россия</t>
+  </si>
+  <si>
     <t>вынос_Одна тонна - Огниво: Cascade &amp; Simcoe, РОЗЛИВ, Россия</t>
   </si>
   <si>
@@ -2022,6 +2037,9 @@
   </si>
   <si>
     <t>Одна тонна - Sunday Draft: Enigma + Idaho 7 (NE Pale Ale), РОЗЛИВ, Россия</t>
+  </si>
+  <si>
+    <t>Одна тонна - Коник (Kolsch), РОЗЛИВ, Россия</t>
   </si>
   <si>
     <t>Одна тонна - Огниво: Cascade &amp; Simcoe, РОЗЛИВ, Россия</t>
@@ -2501,7 +2519,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:B710"/>
+  <dimension ref="A1:B716"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="122.541504" bestFit="true" customWidth="true" style="0"/>
@@ -4233,7 +4251,7 @@
         <v>216</v>
       </c>
       <c r="B216" s="1">
-        <v>640</v>
+        <v>780</v>
       </c>
     </row>
     <row r="217" spans="1:2">
@@ -4249,7 +4267,7 @@
         <v>218</v>
       </c>
       <c r="B218" s="1">
-        <v>1000</v>
+        <v>640</v>
       </c>
     </row>
     <row r="219" spans="1:2">
@@ -4257,7 +4275,7 @@
         <v>219</v>
       </c>
       <c r="B219" s="1">
-        <v>500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="220" spans="1:2">
@@ -4265,7 +4283,7 @@
         <v>220</v>
       </c>
       <c r="B220" s="1">
-        <v>758</v>
+        <v>500</v>
       </c>
     </row>
     <row r="221" spans="1:2">
@@ -4273,7 +4291,7 @@
         <v>221</v>
       </c>
       <c r="B221" s="1">
-        <v>2273</v>
+        <v>758</v>
       </c>
     </row>
     <row r="222" spans="1:2">
@@ -4281,7 +4299,7 @@
         <v>222</v>
       </c>
       <c r="B222" s="1">
-        <v>1515</v>
+        <v>2273</v>
       </c>
     </row>
     <row r="223" spans="1:2">
@@ -4289,7 +4307,7 @@
         <v>223</v>
       </c>
       <c r="B223" s="1">
-        <v>520</v>
+        <v>1515</v>
       </c>
     </row>
     <row r="224" spans="1:2">
@@ -4297,7 +4315,7 @@
         <v>224</v>
       </c>
       <c r="B224" s="1">
-        <v>720</v>
+        <v>520</v>
       </c>
     </row>
     <row r="225" spans="1:2">
@@ -4305,7 +4323,7 @@
         <v>225</v>
       </c>
       <c r="B225" s="1">
-        <v>560</v>
+        <v>720</v>
       </c>
     </row>
     <row r="226" spans="1:2">
@@ -4313,7 +4331,7 @@
         <v>226</v>
       </c>
       <c r="B226" s="1">
-        <v>480</v>
+        <v>560</v>
       </c>
     </row>
     <row r="227" spans="1:2">
@@ -4321,7 +4339,7 @@
         <v>227</v>
       </c>
       <c r="B227" s="1">
-        <v>720</v>
+        <v>480</v>
       </c>
     </row>
     <row r="228" spans="1:2">
@@ -4337,7 +4355,7 @@
         <v>229</v>
       </c>
       <c r="B229" s="1">
-        <v>600</v>
+        <v>720</v>
       </c>
     </row>
     <row r="230" spans="1:2">
@@ -4345,7 +4363,7 @@
         <v>230</v>
       </c>
       <c r="B230" s="1">
-        <v>700</v>
+        <v>600</v>
       </c>
     </row>
     <row r="231" spans="1:2">
@@ -4353,7 +4371,7 @@
         <v>231</v>
       </c>
       <c r="B231" s="1">
-        <v>580</v>
+        <v>700</v>
       </c>
     </row>
     <row r="232" spans="1:2">
@@ -4361,7 +4379,7 @@
         <v>232</v>
       </c>
       <c r="B232" s="1">
-        <v>520</v>
+        <v>580</v>
       </c>
     </row>
     <row r="233" spans="1:2">
@@ -4369,7 +4387,7 @@
         <v>233</v>
       </c>
       <c r="B233" s="1">
-        <v>680</v>
+        <v>520</v>
       </c>
     </row>
     <row r="234" spans="1:2">
@@ -4377,7 +4395,7 @@
         <v>234</v>
       </c>
       <c r="B234" s="1">
-        <v>640</v>
+        <v>680</v>
       </c>
     </row>
     <row r="235" spans="1:2">
@@ -4385,7 +4403,7 @@
         <v>235</v>
       </c>
       <c r="B235" s="1">
-        <v>580</v>
+        <v>640</v>
       </c>
     </row>
     <row r="236" spans="1:2">
@@ -4393,7 +4411,7 @@
         <v>236</v>
       </c>
       <c r="B236" s="1">
-        <v>560</v>
+        <v>580</v>
       </c>
     </row>
     <row r="237" spans="1:2">
@@ -4401,7 +4419,7 @@
         <v>237</v>
       </c>
       <c r="B237" s="1">
-        <v>380</v>
+        <v>560</v>
       </c>
     </row>
     <row r="238" spans="1:2">
@@ -4409,7 +4427,7 @@
         <v>238</v>
       </c>
       <c r="B238" s="1">
-        <v>660</v>
+        <v>380</v>
       </c>
     </row>
     <row r="239" spans="1:2">
@@ -4417,7 +4435,7 @@
         <v>239</v>
       </c>
       <c r="B239" s="1">
-        <v>540</v>
+        <v>660</v>
       </c>
     </row>
     <row r="240" spans="1:2">
@@ -4425,7 +4443,7 @@
         <v>240</v>
       </c>
       <c r="B240" s="1">
-        <v>520</v>
+        <v>540</v>
       </c>
     </row>
     <row r="241" spans="1:2">
@@ -4433,7 +4451,7 @@
         <v>241</v>
       </c>
       <c r="B241" s="1">
-        <v>660</v>
+        <v>520</v>
       </c>
     </row>
     <row r="242" spans="1:2">
@@ -4441,7 +4459,7 @@
         <v>242</v>
       </c>
       <c r="B242" s="1">
-        <v>580</v>
+        <v>660</v>
       </c>
     </row>
     <row r="243" spans="1:2">
@@ -4449,7 +4467,7 @@
         <v>243</v>
       </c>
       <c r="B243" s="1">
-        <v>460</v>
+        <v>580</v>
       </c>
     </row>
     <row r="244" spans="1:2">
@@ -4457,7 +4475,7 @@
         <v>244</v>
       </c>
       <c r="B244" s="1">
-        <v>520</v>
+        <v>460</v>
       </c>
     </row>
     <row r="245" spans="1:2">
@@ -4465,7 +4483,7 @@
         <v>245</v>
       </c>
       <c r="B245" s="1">
-        <v>580</v>
+        <v>520</v>
       </c>
     </row>
     <row r="246" spans="1:2">
@@ -4473,7 +4491,7 @@
         <v>246</v>
       </c>
       <c r="B246" s="1">
-        <v>860</v>
+        <v>580</v>
       </c>
     </row>
     <row r="247" spans="1:2">
@@ -4489,7 +4507,7 @@
         <v>248</v>
       </c>
       <c r="B248" s="1">
-        <v>560</v>
+        <v>860</v>
       </c>
     </row>
     <row r="249" spans="1:2">
@@ -4497,7 +4515,7 @@
         <v>249</v>
       </c>
       <c r="B249" s="1">
-        <v>560</v>
+        <v>900</v>
       </c>
     </row>
     <row r="250" spans="1:2">
@@ -4505,7 +4523,7 @@
         <v>250</v>
       </c>
       <c r="B250" s="1">
-        <v>1000</v>
+        <v>560</v>
       </c>
     </row>
     <row r="251" spans="1:2">
@@ -4513,7 +4531,7 @@
         <v>251</v>
       </c>
       <c r="B251" s="1">
-        <v>900</v>
+        <v>560</v>
       </c>
     </row>
     <row r="252" spans="1:2">
@@ -4521,7 +4539,7 @@
         <v>252</v>
       </c>
       <c r="B252" s="1">
-        <v>680</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="253" spans="1:2">
@@ -4529,7 +4547,7 @@
         <v>253</v>
       </c>
       <c r="B253" s="1">
-        <v>1000</v>
+        <v>900</v>
       </c>
     </row>
     <row r="254" spans="1:2">
@@ -4537,7 +4555,7 @@
         <v>254</v>
       </c>
       <c r="B254" s="1">
-        <v>840</v>
+        <v>680</v>
       </c>
     </row>
     <row r="255" spans="1:2">
@@ -4553,7 +4571,7 @@
         <v>256</v>
       </c>
       <c r="B256" s="1">
-        <v>1020</v>
+        <v>840</v>
       </c>
     </row>
     <row r="257" spans="1:2">
@@ -4569,7 +4587,7 @@
         <v>258</v>
       </c>
       <c r="B258" s="1">
-        <v>680</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="259" spans="1:2">
@@ -4577,7 +4595,7 @@
         <v>259</v>
       </c>
       <c r="B259" s="1">
-        <v>520</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="260" spans="1:2">
@@ -4585,7 +4603,7 @@
         <v>260</v>
       </c>
       <c r="B260" s="1">
-        <v>640</v>
+        <v>680</v>
       </c>
     </row>
     <row r="261" spans="1:2">
@@ -4593,7 +4611,7 @@
         <v>261</v>
       </c>
       <c r="B261" s="1">
-        <v>800</v>
+        <v>520</v>
       </c>
     </row>
     <row r="262" spans="1:2">
@@ -4601,7 +4619,7 @@
         <v>262</v>
       </c>
       <c r="B262" s="1">
-        <v>660</v>
+        <v>640</v>
       </c>
     </row>
     <row r="263" spans="1:2">
@@ -4609,7 +4627,7 @@
         <v>263</v>
       </c>
       <c r="B263" s="1">
-        <v>700</v>
+        <v>800</v>
       </c>
     </row>
     <row r="264" spans="1:2">
@@ -4617,7 +4635,7 @@
         <v>264</v>
       </c>
       <c r="B264" s="1">
-        <v>580</v>
+        <v>660</v>
       </c>
     </row>
     <row r="265" spans="1:2">
@@ -4625,7 +4643,7 @@
         <v>265</v>
       </c>
       <c r="B265" s="1">
-        <v>640</v>
+        <v>700</v>
       </c>
     </row>
     <row r="266" spans="1:2">
@@ -4633,7 +4651,7 @@
         <v>266</v>
       </c>
       <c r="B266" s="1">
-        <v>740</v>
+        <v>580</v>
       </c>
     </row>
     <row r="267" spans="1:2">
@@ -4641,7 +4659,7 @@
         <v>267</v>
       </c>
       <c r="B267" s="1">
-        <v>720</v>
+        <v>640</v>
       </c>
     </row>
     <row r="268" spans="1:2">
@@ -4649,7 +4667,7 @@
         <v>268</v>
       </c>
       <c r="B268" s="1">
-        <v>640</v>
+        <v>740</v>
       </c>
     </row>
     <row r="269" spans="1:2">
@@ -4665,7 +4683,7 @@
         <v>270</v>
       </c>
       <c r="B270" s="1">
-        <v>880</v>
+        <v>640</v>
       </c>
     </row>
     <row r="271" spans="1:2">
@@ -4673,7 +4691,7 @@
         <v>271</v>
       </c>
       <c r="B271" s="1">
-        <v>520</v>
+        <v>720</v>
       </c>
     </row>
     <row r="272" spans="1:2">
@@ -4681,7 +4699,7 @@
         <v>272</v>
       </c>
       <c r="B272" s="1">
-        <v>740</v>
+        <v>880</v>
       </c>
     </row>
     <row r="273" spans="1:2">
@@ -4689,7 +4707,7 @@
         <v>273</v>
       </c>
       <c r="B273" s="1">
-        <v>600</v>
+        <v>520</v>
       </c>
     </row>
     <row r="274" spans="1:2">
@@ -4697,7 +4715,7 @@
         <v>274</v>
       </c>
       <c r="B274" s="1">
-        <v>820</v>
+        <v>740</v>
       </c>
     </row>
     <row r="275" spans="1:2">
@@ -4713,7 +4731,7 @@
         <v>276</v>
       </c>
       <c r="B276" s="1">
-        <v>380</v>
+        <v>820</v>
       </c>
     </row>
     <row r="277" spans="1:2">
@@ -4721,7 +4739,7 @@
         <v>277</v>
       </c>
       <c r="B277" s="1">
-        <v>520</v>
+        <v>600</v>
       </c>
     </row>
     <row r="278" spans="1:2">
@@ -4729,7 +4747,7 @@
         <v>278</v>
       </c>
       <c r="B278" s="1">
-        <v>320</v>
+        <v>380</v>
       </c>
     </row>
     <row r="279" spans="1:2">
@@ -4737,7 +4755,7 @@
         <v>279</v>
       </c>
       <c r="B279" s="1">
-        <v>540</v>
+        <v>520</v>
       </c>
     </row>
     <row r="280" spans="1:2">
@@ -4745,7 +4763,7 @@
         <v>280</v>
       </c>
       <c r="B280" s="1">
-        <v>560</v>
+        <v>320</v>
       </c>
     </row>
     <row r="281" spans="1:2">
@@ -4753,7 +4771,7 @@
         <v>281</v>
       </c>
       <c r="B281" s="1">
-        <v>480</v>
+        <v>540</v>
       </c>
     </row>
     <row r="282" spans="1:2">
@@ -4761,7 +4779,7 @@
         <v>282</v>
       </c>
       <c r="B282" s="1">
-        <v>480</v>
+        <v>560</v>
       </c>
     </row>
     <row r="283" spans="1:2">
@@ -4769,7 +4787,7 @@
         <v>283</v>
       </c>
       <c r="B283" s="1">
-        <v>520</v>
+        <v>480</v>
       </c>
     </row>
     <row r="284" spans="1:2">
@@ -4777,7 +4795,7 @@
         <v>284</v>
       </c>
       <c r="B284" s="1">
-        <v>500</v>
+        <v>480</v>
       </c>
     </row>
     <row r="285" spans="1:2">
@@ -4785,7 +4803,7 @@
         <v>285</v>
       </c>
       <c r="B285" s="1">
-        <v>640</v>
+        <v>520</v>
       </c>
     </row>
     <row r="286" spans="1:2">
@@ -4793,7 +4811,7 @@
         <v>286</v>
       </c>
       <c r="B286" s="1">
-        <v>480</v>
+        <v>500</v>
       </c>
     </row>
     <row r="287" spans="1:2">
@@ -4801,7 +4819,7 @@
         <v>287</v>
       </c>
       <c r="B287" s="1">
-        <v>740</v>
+        <v>640</v>
       </c>
     </row>
     <row r="288" spans="1:2">
@@ -4809,7 +4827,7 @@
         <v>288</v>
       </c>
       <c r="B288" s="1">
-        <v>520</v>
+        <v>480</v>
       </c>
     </row>
     <row r="289" spans="1:2">
@@ -4817,7 +4835,7 @@
         <v>289</v>
       </c>
       <c r="B289" s="1">
-        <v>380</v>
+        <v>780</v>
       </c>
     </row>
     <row r="290" spans="1:2">
@@ -4825,7 +4843,7 @@
         <v>290</v>
       </c>
       <c r="B290" s="1">
-        <v>440</v>
+        <v>520</v>
       </c>
     </row>
     <row r="291" spans="1:2">
@@ -4833,7 +4851,7 @@
         <v>291</v>
       </c>
       <c r="B291" s="1">
-        <v>900</v>
+        <v>380</v>
       </c>
     </row>
     <row r="292" spans="1:2">
@@ -4841,7 +4859,7 @@
         <v>292</v>
       </c>
       <c r="B292" s="1">
-        <v>900</v>
+        <v>440</v>
       </c>
     </row>
     <row r="293" spans="1:2">
@@ -4849,7 +4867,7 @@
         <v>293</v>
       </c>
       <c r="B293" s="1">
-        <v>720</v>
+        <v>900</v>
       </c>
     </row>
     <row r="294" spans="1:2">
@@ -4857,7 +4875,7 @@
         <v>294</v>
       </c>
       <c r="B294" s="1">
-        <v>960</v>
+        <v>900</v>
       </c>
     </row>
     <row r="295" spans="1:2">
@@ -4865,7 +4883,7 @@
         <v>295</v>
       </c>
       <c r="B295" s="1">
-        <v>1020</v>
+        <v>720</v>
       </c>
     </row>
     <row r="296" spans="1:2">
@@ -4873,7 +4891,7 @@
         <v>296</v>
       </c>
       <c r="B296" s="1">
-        <v>780</v>
+        <v>960</v>
       </c>
     </row>
     <row r="297" spans="1:2">
@@ -4881,7 +4899,7 @@
         <v>297</v>
       </c>
       <c r="B297" s="1">
-        <v>700</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="298" spans="1:2">
@@ -4889,7 +4907,7 @@
         <v>298</v>
       </c>
       <c r="B298" s="1">
-        <v>640</v>
+        <v>780</v>
       </c>
     </row>
     <row r="299" spans="1:2">
@@ -4897,7 +4915,7 @@
         <v>299</v>
       </c>
       <c r="B299" s="1">
-        <v>780</v>
+        <v>700</v>
       </c>
     </row>
     <row r="300" spans="1:2">
@@ -4905,7 +4923,7 @@
         <v>300</v>
       </c>
       <c r="B300" s="1">
-        <v>1020</v>
+        <v>640</v>
       </c>
     </row>
     <row r="301" spans="1:2">
@@ -4921,7 +4939,7 @@
         <v>302</v>
       </c>
       <c r="B302" s="1">
-        <v>1000</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="303" spans="1:2">
@@ -4929,7 +4947,7 @@
         <v>303</v>
       </c>
       <c r="B303" s="1">
-        <v>1000</v>
+        <v>780</v>
       </c>
     </row>
     <row r="304" spans="1:2">
@@ -4937,7 +4955,7 @@
         <v>304</v>
       </c>
       <c r="B304" s="1">
-        <v>780</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="305" spans="1:2">
@@ -4945,7 +4963,7 @@
         <v>305</v>
       </c>
       <c r="B305" s="1">
-        <v>720</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="306" spans="1:2">
@@ -4953,7 +4971,7 @@
         <v>306</v>
       </c>
       <c r="B306" s="1">
-        <v>680</v>
+        <v>780</v>
       </c>
     </row>
     <row r="307" spans="1:2">
@@ -4961,7 +4979,7 @@
         <v>307</v>
       </c>
       <c r="B307" s="1">
-        <v>700</v>
+        <v>720</v>
       </c>
     </row>
     <row r="308" spans="1:2">
@@ -4977,7 +4995,7 @@
         <v>309</v>
       </c>
       <c r="B309" s="1">
-        <v>740</v>
+        <v>700</v>
       </c>
     </row>
     <row r="310" spans="1:2">
@@ -4985,7 +5003,7 @@
         <v>310</v>
       </c>
       <c r="B310" s="1">
-        <v>740</v>
+        <v>680</v>
       </c>
     </row>
     <row r="311" spans="1:2">
@@ -4993,7 +5011,7 @@
         <v>311</v>
       </c>
       <c r="B311" s="1">
-        <v>680</v>
+        <v>740</v>
       </c>
     </row>
     <row r="312" spans="1:2">
@@ -5001,7 +5019,7 @@
         <v>312</v>
       </c>
       <c r="B312" s="1">
-        <v>480</v>
+        <v>740</v>
       </c>
     </row>
     <row r="313" spans="1:2">
@@ -5009,7 +5027,7 @@
         <v>313</v>
       </c>
       <c r="B313" s="1">
-        <v>640</v>
+        <v>680</v>
       </c>
     </row>
     <row r="314" spans="1:2">
@@ -5017,7 +5035,7 @@
         <v>314</v>
       </c>
       <c r="B314" s="1">
-        <v>1000</v>
+        <v>480</v>
       </c>
     </row>
     <row r="315" spans="1:2">
@@ -5025,7 +5043,7 @@
         <v>315</v>
       </c>
       <c r="B315" s="1">
-        <v>920</v>
+        <v>640</v>
       </c>
     </row>
     <row r="316" spans="1:2">
@@ -5033,7 +5051,7 @@
         <v>316</v>
       </c>
       <c r="B316" s="1">
-        <v>860</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="317" spans="1:2">
@@ -5041,7 +5059,7 @@
         <v>317</v>
       </c>
       <c r="B317" s="1">
-        <v>520</v>
+        <v>920</v>
       </c>
     </row>
     <row r="318" spans="1:2">
@@ -5049,7 +5067,7 @@
         <v>318</v>
       </c>
       <c r="B318" s="1">
-        <v>540</v>
+        <v>860</v>
       </c>
     </row>
     <row r="319" spans="1:2">
@@ -5057,7 +5075,7 @@
         <v>319</v>
       </c>
       <c r="B319" s="1">
-        <v>700</v>
+        <v>520</v>
       </c>
     </row>
     <row r="320" spans="1:2">
@@ -5065,7 +5083,7 @@
         <v>320</v>
       </c>
       <c r="B320" s="1">
-        <v>700</v>
+        <v>540</v>
       </c>
     </row>
     <row r="321" spans="1:2">
@@ -5073,7 +5091,7 @@
         <v>321</v>
       </c>
       <c r="B321" s="1">
-        <v>420</v>
+        <v>700</v>
       </c>
     </row>
     <row r="322" spans="1:2">
@@ -5089,7 +5107,7 @@
         <v>323</v>
       </c>
       <c r="B323" s="1">
-        <v>720</v>
+        <v>420</v>
       </c>
     </row>
     <row r="324" spans="1:2">
@@ -5097,7 +5115,7 @@
         <v>324</v>
       </c>
       <c r="B324" s="1">
-        <v>580</v>
+        <v>700</v>
       </c>
     </row>
     <row r="325" spans="1:2">
@@ -5105,7 +5123,7 @@
         <v>325</v>
       </c>
       <c r="B325" s="1">
-        <v>740</v>
+        <v>720</v>
       </c>
     </row>
     <row r="326" spans="1:2">
@@ -5113,7 +5131,7 @@
         <v>326</v>
       </c>
       <c r="B326" s="1">
-        <v>900</v>
+        <v>580</v>
       </c>
     </row>
     <row r="327" spans="1:2">
@@ -5121,7 +5139,7 @@
         <v>327</v>
       </c>
       <c r="B327" s="1">
-        <v>920</v>
+        <v>740</v>
       </c>
     </row>
     <row r="328" spans="1:2">
@@ -5129,7 +5147,7 @@
         <v>328</v>
       </c>
       <c r="B328" s="1">
-        <v>840</v>
+        <v>900</v>
       </c>
     </row>
     <row r="329" spans="1:2">
@@ -5137,7 +5155,7 @@
         <v>329</v>
       </c>
       <c r="B329" s="1">
-        <v>720</v>
+        <v>920</v>
       </c>
     </row>
     <row r="330" spans="1:2">
@@ -5145,7 +5163,7 @@
         <v>330</v>
       </c>
       <c r="B330" s="1">
-        <v>620</v>
+        <v>840</v>
       </c>
     </row>
     <row r="331" spans="1:2">
@@ -5153,7 +5171,7 @@
         <v>331</v>
       </c>
       <c r="B331" s="1">
-        <v>440</v>
+        <v>720</v>
       </c>
     </row>
     <row r="332" spans="1:2">
@@ -5161,7 +5179,7 @@
         <v>332</v>
       </c>
       <c r="B332" s="1">
-        <v>320</v>
+        <v>620</v>
       </c>
     </row>
     <row r="333" spans="1:2">
@@ -5169,7 +5187,7 @@
         <v>333</v>
       </c>
       <c r="B333" s="1">
-        <v>320</v>
+        <v>440</v>
       </c>
     </row>
     <row r="334" spans="1:2">
@@ -5177,7 +5195,7 @@
         <v>334</v>
       </c>
       <c r="B334" s="1">
-        <v>820</v>
+        <v>320</v>
       </c>
     </row>
     <row r="335" spans="1:2">
@@ -5185,7 +5203,7 @@
         <v>335</v>
       </c>
       <c r="B335" s="1">
-        <v>1000</v>
+        <v>320</v>
       </c>
     </row>
     <row r="336" spans="1:2">
@@ -5193,7 +5211,7 @@
         <v>336</v>
       </c>
       <c r="B336" s="1">
-        <v>580</v>
+        <v>820</v>
       </c>
     </row>
     <row r="337" spans="1:2">
@@ -5201,7 +5219,7 @@
         <v>337</v>
       </c>
       <c r="B337" s="1">
-        <v>580</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="338" spans="1:2">
@@ -5209,7 +5227,7 @@
         <v>338</v>
       </c>
       <c r="B338" s="1">
-        <v>900</v>
+        <v>580</v>
       </c>
     </row>
     <row r="339" spans="1:2">
@@ -5225,7 +5243,7 @@
         <v>340</v>
       </c>
       <c r="B340" s="1">
-        <v>580</v>
+        <v>900</v>
       </c>
     </row>
     <row r="341" spans="1:2">
@@ -5233,7 +5251,7 @@
         <v>341</v>
       </c>
       <c r="B341" s="1">
-        <v>620</v>
+        <v>580</v>
       </c>
     </row>
     <row r="342" spans="1:2">
@@ -5241,7 +5259,7 @@
         <v>342</v>
       </c>
       <c r="B342" s="1">
-        <v>900</v>
+        <v>580</v>
       </c>
     </row>
     <row r="343" spans="1:2">
@@ -5249,7 +5267,7 @@
         <v>343</v>
       </c>
       <c r="B343" s="1">
-        <v>1000</v>
+        <v>620</v>
       </c>
     </row>
     <row r="344" spans="1:2">
@@ -5257,7 +5275,7 @@
         <v>344</v>
       </c>
       <c r="B344" s="1">
-        <v>780</v>
+        <v>900</v>
       </c>
     </row>
     <row r="345" spans="1:2">
@@ -5265,7 +5283,7 @@
         <v>345</v>
       </c>
       <c r="B345" s="1">
-        <v>880</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="346" spans="1:2">
@@ -5281,7 +5299,7 @@
         <v>347</v>
       </c>
       <c r="B347" s="1">
-        <v>740</v>
+        <v>880</v>
       </c>
     </row>
     <row r="348" spans="1:2">
@@ -5289,7 +5307,7 @@
         <v>348</v>
       </c>
       <c r="B348" s="1">
-        <v>900</v>
+        <v>780</v>
       </c>
     </row>
     <row r="349" spans="1:2">
@@ -5297,7 +5315,7 @@
         <v>349</v>
       </c>
       <c r="B349" s="1">
-        <v>660</v>
+        <v>740</v>
       </c>
     </row>
     <row r="350" spans="1:2">
@@ -5305,7 +5323,7 @@
         <v>350</v>
       </c>
       <c r="B350" s="1">
-        <v>700</v>
+        <v>900</v>
       </c>
     </row>
     <row r="351" spans="1:2">
@@ -5313,7 +5331,7 @@
         <v>351</v>
       </c>
       <c r="B351" s="1">
-        <v>680</v>
+        <v>660</v>
       </c>
     </row>
     <row r="352" spans="1:2">
@@ -5321,7 +5339,7 @@
         <v>352</v>
       </c>
       <c r="B352" s="1">
-        <v>660</v>
+        <v>700</v>
       </c>
     </row>
     <row r="353" spans="1:2">
@@ -5329,7 +5347,7 @@
         <v>353</v>
       </c>
       <c r="B353" s="1">
-        <v>440</v>
+        <v>680</v>
       </c>
     </row>
     <row r="354" spans="1:2">
@@ -5337,7 +5355,7 @@
         <v>354</v>
       </c>
       <c r="B354" s="1">
-        <v>700</v>
+        <v>660</v>
       </c>
     </row>
     <row r="355" spans="1:2">
@@ -5345,7 +5363,7 @@
         <v>355</v>
       </c>
       <c r="B355" s="1">
-        <v>800</v>
+        <v>440</v>
       </c>
     </row>
     <row r="356" spans="1:2">
@@ -5353,7 +5371,7 @@
         <v>356</v>
       </c>
       <c r="B356" s="1">
-        <v>560</v>
+        <v>700</v>
       </c>
     </row>
     <row r="357" spans="1:2">
@@ -5361,7 +5379,7 @@
         <v>357</v>
       </c>
       <c r="B357" s="1">
-        <v>760</v>
+        <v>800</v>
       </c>
     </row>
     <row r="358" spans="1:2">
@@ -5369,7 +5387,7 @@
         <v>358</v>
       </c>
       <c r="B358" s="1">
-        <v>780</v>
+        <v>560</v>
       </c>
     </row>
     <row r="359" spans="1:2">
@@ -5377,7 +5395,7 @@
         <v>359</v>
       </c>
       <c r="B359" s="1">
-        <v>720</v>
+        <v>760</v>
       </c>
     </row>
     <row r="360" spans="1:2">
@@ -5385,7 +5403,7 @@
         <v>360</v>
       </c>
       <c r="B360" s="1">
-        <v>600</v>
+        <v>780</v>
       </c>
     </row>
     <row r="361" spans="1:2">
@@ -5393,7 +5411,7 @@
         <v>361</v>
       </c>
       <c r="B361" s="1">
-        <v>560</v>
+        <v>720</v>
       </c>
     </row>
     <row r="362" spans="1:2">
@@ -5401,7 +5419,7 @@
         <v>362</v>
       </c>
       <c r="B362" s="1">
-        <v>620</v>
+        <v>600</v>
       </c>
     </row>
     <row r="363" spans="1:2">
@@ -5409,7 +5427,7 @@
         <v>363</v>
       </c>
       <c r="B363" s="1">
-        <v>720</v>
+        <v>560</v>
       </c>
     </row>
     <row r="364" spans="1:2">
@@ -5417,7 +5435,7 @@
         <v>364</v>
       </c>
       <c r="B364" s="1">
-        <v>680</v>
+        <v>620</v>
       </c>
     </row>
     <row r="365" spans="1:2">
@@ -5425,7 +5443,7 @@
         <v>365</v>
       </c>
       <c r="B365" s="1">
-        <v>480</v>
+        <v>720</v>
       </c>
     </row>
     <row r="366" spans="1:2">
@@ -5433,7 +5451,7 @@
         <v>366</v>
       </c>
       <c r="B366" s="1">
-        <v>480</v>
+        <v>680</v>
       </c>
     </row>
     <row r="367" spans="1:2">
@@ -5441,7 +5459,7 @@
         <v>367</v>
       </c>
       <c r="B367" s="1">
-        <v>900</v>
+        <v>480</v>
       </c>
     </row>
     <row r="368" spans="1:2">
@@ -5449,7 +5467,7 @@
         <v>368</v>
       </c>
       <c r="B368" s="1">
-        <v>800</v>
+        <v>480</v>
       </c>
     </row>
     <row r="369" spans="1:2">
@@ -5457,7 +5475,7 @@
         <v>369</v>
       </c>
       <c r="B369" s="1">
-        <v>780</v>
+        <v>900</v>
       </c>
     </row>
     <row r="370" spans="1:2">
@@ -5465,7 +5483,7 @@
         <v>370</v>
       </c>
       <c r="B370" s="1">
-        <v>920</v>
+        <v>800</v>
       </c>
     </row>
     <row r="371" spans="1:2">
@@ -5473,7 +5491,7 @@
         <v>371</v>
       </c>
       <c r="B371" s="1">
-        <v>740</v>
+        <v>780</v>
       </c>
     </row>
     <row r="372" spans="1:2">
@@ -5481,7 +5499,7 @@
         <v>372</v>
       </c>
       <c r="B372" s="1">
-        <v>740</v>
+        <v>920</v>
       </c>
     </row>
     <row r="373" spans="1:2">
@@ -5489,7 +5507,7 @@
         <v>373</v>
       </c>
       <c r="B373" s="1">
-        <v>940</v>
+        <v>740</v>
       </c>
     </row>
     <row r="374" spans="1:2">
@@ -5497,7 +5515,7 @@
         <v>374</v>
       </c>
       <c r="B374" s="1">
-        <v>980</v>
+        <v>740</v>
       </c>
     </row>
     <row r="375" spans="1:2">
@@ -5505,7 +5523,7 @@
         <v>375</v>
       </c>
       <c r="B375" s="1">
-        <v>920</v>
+        <v>940</v>
       </c>
     </row>
     <row r="376" spans="1:2">
@@ -5513,7 +5531,7 @@
         <v>376</v>
       </c>
       <c r="B376" s="1">
-        <v>600</v>
+        <v>980</v>
       </c>
     </row>
     <row r="377" spans="1:2">
@@ -5521,7 +5539,7 @@
         <v>377</v>
       </c>
       <c r="B377" s="1">
-        <v>760</v>
+        <v>920</v>
       </c>
     </row>
     <row r="378" spans="1:2">
@@ -5529,7 +5547,7 @@
         <v>378</v>
       </c>
       <c r="B378" s="1">
-        <v>780</v>
+        <v>600</v>
       </c>
     </row>
     <row r="379" spans="1:2">
@@ -5537,7 +5555,7 @@
         <v>379</v>
       </c>
       <c r="B379" s="1">
-        <v>620</v>
+        <v>760</v>
       </c>
     </row>
     <row r="380" spans="1:2">
@@ -5545,7 +5563,7 @@
         <v>380</v>
       </c>
       <c r="B380" s="1">
-        <v>620</v>
+        <v>780</v>
       </c>
     </row>
     <row r="381" spans="1:2">
@@ -5553,7 +5571,7 @@
         <v>381</v>
       </c>
       <c r="B381" s="1">
-        <v>860</v>
+        <v>620</v>
       </c>
     </row>
     <row r="382" spans="1:2">
@@ -5561,7 +5579,7 @@
         <v>382</v>
       </c>
       <c r="B382" s="1">
-        <v>920</v>
+        <v>620</v>
       </c>
     </row>
     <row r="383" spans="1:2">
@@ -5569,7 +5587,7 @@
         <v>383</v>
       </c>
       <c r="B383" s="1">
-        <v>640</v>
+        <v>860</v>
       </c>
     </row>
     <row r="384" spans="1:2">
@@ -5577,7 +5595,7 @@
         <v>384</v>
       </c>
       <c r="B384" s="1">
-        <v>680</v>
+        <v>920</v>
       </c>
     </row>
     <row r="385" spans="1:2">
@@ -5585,7 +5603,7 @@
         <v>385</v>
       </c>
       <c r="B385" s="1">
-        <v>820</v>
+        <v>640</v>
       </c>
     </row>
     <row r="386" spans="1:2">
@@ -5593,7 +5611,7 @@
         <v>386</v>
       </c>
       <c r="B386" s="1">
-        <v>960</v>
+        <v>680</v>
       </c>
     </row>
     <row r="387" spans="1:2">
@@ -5601,7 +5619,7 @@
         <v>387</v>
       </c>
       <c r="B387" s="1">
-        <v>740</v>
+        <v>820</v>
       </c>
     </row>
     <row r="388" spans="1:2">
@@ -5609,7 +5627,7 @@
         <v>388</v>
       </c>
       <c r="B388" s="1">
-        <v>1000</v>
+        <v>960</v>
       </c>
     </row>
     <row r="389" spans="1:2">
@@ -5617,7 +5635,7 @@
         <v>389</v>
       </c>
       <c r="B389" s="1">
-        <v>640</v>
+        <v>740</v>
       </c>
     </row>
     <row r="390" spans="1:2">
@@ -5625,7 +5643,7 @@
         <v>390</v>
       </c>
       <c r="B390" s="1">
-        <v>860</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="391" spans="1:2">
@@ -5633,7 +5651,7 @@
         <v>391</v>
       </c>
       <c r="B391" s="1">
-        <v>560</v>
+        <v>640</v>
       </c>
     </row>
     <row r="392" spans="1:2">
@@ -5641,7 +5659,7 @@
         <v>392</v>
       </c>
       <c r="B392" s="1">
-        <v>780</v>
+        <v>860</v>
       </c>
     </row>
     <row r="393" spans="1:2">
@@ -5649,7 +5667,7 @@
         <v>393</v>
       </c>
       <c r="B393" s="1">
-        <v>660</v>
+        <v>560</v>
       </c>
     </row>
     <row r="394" spans="1:2">
@@ -5657,7 +5675,7 @@
         <v>394</v>
       </c>
       <c r="B394" s="1">
-        <v>640</v>
+        <v>780</v>
       </c>
     </row>
     <row r="395" spans="1:2">
@@ -5665,7 +5683,7 @@
         <v>395</v>
       </c>
       <c r="B395" s="1">
-        <v>560</v>
+        <v>660</v>
       </c>
     </row>
     <row r="396" spans="1:2">
@@ -5673,7 +5691,7 @@
         <v>396</v>
       </c>
       <c r="B396" s="1">
-        <v>840</v>
+        <v>640</v>
       </c>
     </row>
     <row r="397" spans="1:2">
@@ -5681,7 +5699,7 @@
         <v>397</v>
       </c>
       <c r="B397" s="1">
-        <v>520</v>
+        <v>560</v>
       </c>
     </row>
     <row r="398" spans="1:2">
@@ -5689,7 +5707,7 @@
         <v>398</v>
       </c>
       <c r="B398" s="1">
-        <v>480</v>
+        <v>840</v>
       </c>
     </row>
     <row r="399" spans="1:2">
@@ -5697,7 +5715,7 @@
         <v>399</v>
       </c>
       <c r="B399" s="1">
-        <v>620</v>
+        <v>520</v>
       </c>
     </row>
     <row r="400" spans="1:2">
@@ -5705,7 +5723,7 @@
         <v>400</v>
       </c>
       <c r="B400" s="1">
-        <v>780</v>
+        <v>480</v>
       </c>
     </row>
     <row r="401" spans="1:2">
@@ -5713,7 +5731,7 @@
         <v>401</v>
       </c>
       <c r="B401" s="1">
-        <v>560</v>
+        <v>620</v>
       </c>
     </row>
     <row r="402" spans="1:2">
@@ -5721,7 +5739,7 @@
         <v>402</v>
       </c>
       <c r="B402" s="1">
-        <v>820</v>
+        <v>780</v>
       </c>
     </row>
     <row r="403" spans="1:2">
@@ -5729,7 +5747,7 @@
         <v>403</v>
       </c>
       <c r="B403" s="1">
-        <v>760</v>
+        <v>560</v>
       </c>
     </row>
     <row r="404" spans="1:2">
@@ -5737,7 +5755,7 @@
         <v>404</v>
       </c>
       <c r="B404" s="1">
-        <v>740</v>
+        <v>820</v>
       </c>
     </row>
     <row r="405" spans="1:2">
@@ -5745,7 +5763,7 @@
         <v>405</v>
       </c>
       <c r="B405" s="1">
-        <v>780</v>
+        <v>760</v>
       </c>
     </row>
     <row r="406" spans="1:2">
@@ -5753,7 +5771,7 @@
         <v>406</v>
       </c>
       <c r="B406" s="1">
-        <v>600</v>
+        <v>740</v>
       </c>
     </row>
     <row r="407" spans="1:2">
@@ -5761,7 +5779,7 @@
         <v>407</v>
       </c>
       <c r="B407" s="1">
-        <v>480</v>
+        <v>780</v>
       </c>
     </row>
     <row r="408" spans="1:2">
@@ -5769,7 +5787,7 @@
         <v>408</v>
       </c>
       <c r="B408" s="1">
-        <v>840</v>
+        <v>600</v>
       </c>
     </row>
     <row r="409" spans="1:2">
@@ -5777,7 +5795,7 @@
         <v>409</v>
       </c>
       <c r="B409" s="1">
-        <v>660</v>
+        <v>480</v>
       </c>
     </row>
     <row r="410" spans="1:2">
@@ -5785,7 +5803,7 @@
         <v>410</v>
       </c>
       <c r="B410" s="1">
-        <v>700</v>
+        <v>840</v>
       </c>
     </row>
     <row r="411" spans="1:2">
@@ -5793,7 +5811,7 @@
         <v>411</v>
       </c>
       <c r="B411" s="1">
-        <v>440</v>
+        <v>660</v>
       </c>
     </row>
     <row r="412" spans="1:2">
@@ -5801,7 +5819,7 @@
         <v>412</v>
       </c>
       <c r="B412" s="1">
-        <v>440</v>
+        <v>700</v>
       </c>
     </row>
     <row r="413" spans="1:2">
@@ -5809,7 +5827,7 @@
         <v>413</v>
       </c>
       <c r="B413" s="1">
-        <v>740</v>
+        <v>440</v>
       </c>
     </row>
     <row r="414" spans="1:2">
@@ -5817,7 +5835,7 @@
         <v>414</v>
       </c>
       <c r="B414" s="1">
-        <v>880</v>
+        <v>440</v>
       </c>
     </row>
     <row r="415" spans="1:2">
@@ -5825,7 +5843,7 @@
         <v>415</v>
       </c>
       <c r="B415" s="1">
-        <v>880</v>
+        <v>740</v>
       </c>
     </row>
     <row r="416" spans="1:2">
@@ -5833,7 +5851,7 @@
         <v>416</v>
       </c>
       <c r="B416" s="1">
-        <v>760</v>
+        <v>880</v>
       </c>
     </row>
     <row r="417" spans="1:2">
@@ -5841,7 +5859,7 @@
         <v>417</v>
       </c>
       <c r="B417" s="1">
-        <v>840</v>
+        <v>880</v>
       </c>
     </row>
     <row r="418" spans="1:2">
@@ -5849,7 +5867,7 @@
         <v>418</v>
       </c>
       <c r="B418" s="1">
-        <v>660</v>
+        <v>760</v>
       </c>
     </row>
     <row r="419" spans="1:2">
@@ -5857,7 +5875,7 @@
         <v>419</v>
       </c>
       <c r="B419" s="1">
-        <v>1100</v>
+        <v>840</v>
       </c>
     </row>
     <row r="420" spans="1:2">
@@ -5865,7 +5883,7 @@
         <v>420</v>
       </c>
       <c r="B420" s="1">
-        <v>840</v>
+        <v>660</v>
       </c>
     </row>
     <row r="421" spans="1:2">
@@ -5873,7 +5891,7 @@
         <v>421</v>
       </c>
       <c r="B421" s="1">
-        <v>700</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="422" spans="1:2">
@@ -5881,7 +5899,7 @@
         <v>422</v>
       </c>
       <c r="B422" s="1">
-        <v>700</v>
+        <v>840</v>
       </c>
     </row>
     <row r="423" spans="1:2">
@@ -5889,7 +5907,7 @@
         <v>423</v>
       </c>
       <c r="B423" s="1">
-        <v>800</v>
+        <v>700</v>
       </c>
     </row>
     <row r="424" spans="1:2">
@@ -5897,7 +5915,7 @@
         <v>424</v>
       </c>
       <c r="B424" s="1">
-        <v>660</v>
+        <v>700</v>
       </c>
     </row>
     <row r="425" spans="1:2">
@@ -5905,7 +5923,7 @@
         <v>425</v>
       </c>
       <c r="B425" s="1">
-        <v>660</v>
+        <v>800</v>
       </c>
     </row>
     <row r="426" spans="1:2">
@@ -5913,7 +5931,7 @@
         <v>426</v>
       </c>
       <c r="B426" s="1">
-        <v>780</v>
+        <v>660</v>
       </c>
     </row>
     <row r="427" spans="1:2">
@@ -5921,7 +5939,7 @@
         <v>427</v>
       </c>
       <c r="B427" s="1">
-        <v>700</v>
+        <v>660</v>
       </c>
     </row>
     <row r="428" spans="1:2">
@@ -5929,7 +5947,7 @@
         <v>428</v>
       </c>
       <c r="B428" s="1">
-        <v>700</v>
+        <v>780</v>
       </c>
     </row>
     <row r="429" spans="1:2">
@@ -5945,7 +5963,7 @@
         <v>430</v>
       </c>
       <c r="B430" s="1">
-        <v>860</v>
+        <v>700</v>
       </c>
     </row>
     <row r="431" spans="1:2">
@@ -5953,7 +5971,7 @@
         <v>431</v>
       </c>
       <c r="B431" s="1">
-        <v>600</v>
+        <v>700</v>
       </c>
     </row>
     <row r="432" spans="1:2">
@@ -5961,7 +5979,7 @@
         <v>432</v>
       </c>
       <c r="B432" s="1">
-        <v>600</v>
+        <v>860</v>
       </c>
     </row>
     <row r="433" spans="1:2">
@@ -5969,7 +5987,7 @@
         <v>433</v>
       </c>
       <c r="B433" s="1">
-        <v>800</v>
+        <v>600</v>
       </c>
     </row>
     <row r="434" spans="1:2">
@@ -5977,7 +5995,7 @@
         <v>434</v>
       </c>
       <c r="B434" s="1">
-        <v>660</v>
+        <v>600</v>
       </c>
     </row>
     <row r="435" spans="1:2">
@@ -5985,7 +6003,7 @@
         <v>435</v>
       </c>
       <c r="B435" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="436" spans="1:2">
@@ -5993,7 +6011,7 @@
         <v>436</v>
       </c>
       <c r="B436" s="1">
-        <v>620</v>
+        <v>660</v>
       </c>
     </row>
     <row r="437" spans="1:2">
@@ -6001,7 +6019,7 @@
         <v>437</v>
       </c>
       <c r="B437" s="1">
-        <v>880</v>
+        <v>600</v>
       </c>
     </row>
     <row r="438" spans="1:2">
@@ -6009,7 +6027,7 @@
         <v>438</v>
       </c>
       <c r="B438" s="1">
-        <v>860</v>
+        <v>620</v>
       </c>
     </row>
     <row r="439" spans="1:2">
@@ -6017,7 +6035,7 @@
         <v>439</v>
       </c>
       <c r="B439" s="1">
-        <v>860</v>
+        <v>880</v>
       </c>
     </row>
     <row r="440" spans="1:2">
@@ -6025,7 +6043,7 @@
         <v>440</v>
       </c>
       <c r="B440" s="1">
-        <v>760</v>
+        <v>860</v>
       </c>
     </row>
     <row r="441" spans="1:2">
@@ -6033,7 +6051,7 @@
         <v>441</v>
       </c>
       <c r="B441" s="1">
-        <v>720</v>
+        <v>860</v>
       </c>
     </row>
     <row r="442" spans="1:2">
@@ -6041,7 +6059,7 @@
         <v>442</v>
       </c>
       <c r="B442" s="1">
-        <v>900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="443" spans="1:2">
@@ -6049,7 +6067,7 @@
         <v>443</v>
       </c>
       <c r="B443" s="1">
-        <v>740</v>
+        <v>720</v>
       </c>
     </row>
     <row r="444" spans="1:2">
@@ -6057,7 +6075,7 @@
         <v>444</v>
       </c>
       <c r="B444" s="1">
-        <v>640</v>
+        <v>900</v>
       </c>
     </row>
     <row r="445" spans="1:2">
@@ -6065,7 +6083,7 @@
         <v>445</v>
       </c>
       <c r="B445" s="1">
-        <v>800</v>
+        <v>740</v>
       </c>
     </row>
     <row r="446" spans="1:2">
@@ -6073,7 +6091,7 @@
         <v>446</v>
       </c>
       <c r="B446" s="1">
-        <v>660</v>
+        <v>640</v>
       </c>
     </row>
     <row r="447" spans="1:2">
@@ -6081,7 +6099,7 @@
         <v>447</v>
       </c>
       <c r="B447" s="1">
-        <v>700</v>
+        <v>800</v>
       </c>
     </row>
     <row r="448" spans="1:2">
@@ -6089,7 +6107,7 @@
         <v>448</v>
       </c>
       <c r="B448" s="1">
-        <v>700</v>
+        <v>660</v>
       </c>
     </row>
     <row r="449" spans="1:2">
@@ -6097,7 +6115,7 @@
         <v>449</v>
       </c>
       <c r="B449" s="1">
-        <v>820</v>
+        <v>700</v>
       </c>
     </row>
     <row r="450" spans="1:2">
@@ -6105,7 +6123,7 @@
         <v>450</v>
       </c>
       <c r="B450" s="1">
-        <v>760</v>
+        <v>700</v>
       </c>
     </row>
     <row r="451" spans="1:2">
@@ -6129,7 +6147,7 @@
         <v>453</v>
       </c>
       <c r="B453" s="1">
-        <v>920</v>
+        <v>820</v>
       </c>
     </row>
     <row r="454" spans="1:2">
@@ -6137,7 +6155,7 @@
         <v>454</v>
       </c>
       <c r="B454" s="1">
-        <v>600</v>
+        <v>760</v>
       </c>
     </row>
     <row r="455" spans="1:2">
@@ -6145,7 +6163,7 @@
         <v>455</v>
       </c>
       <c r="B455" s="1">
-        <v>880</v>
+        <v>920</v>
       </c>
     </row>
     <row r="456" spans="1:2">
@@ -6153,7 +6171,7 @@
         <v>456</v>
       </c>
       <c r="B456" s="1">
-        <v>640</v>
+        <v>600</v>
       </c>
     </row>
     <row r="457" spans="1:2">
@@ -6161,7 +6179,7 @@
         <v>457</v>
       </c>
       <c r="B457" s="1">
-        <v>700</v>
+        <v>880</v>
       </c>
     </row>
     <row r="458" spans="1:2">
@@ -6169,7 +6187,7 @@
         <v>458</v>
       </c>
       <c r="B458" s="1">
-        <v>600</v>
+        <v>640</v>
       </c>
     </row>
     <row r="459" spans="1:2">
@@ -6177,7 +6195,7 @@
         <v>459</v>
       </c>
       <c r="B459" s="1">
-        <v>560</v>
+        <v>700</v>
       </c>
     </row>
     <row r="460" spans="1:2">
@@ -6185,7 +6203,7 @@
         <v>460</v>
       </c>
       <c r="B460" s="1">
-        <v>560</v>
+        <v>600</v>
       </c>
     </row>
     <row r="461" spans="1:2">
@@ -6193,7 +6211,7 @@
         <v>461</v>
       </c>
       <c r="B461" s="1">
-        <v>860</v>
+        <v>560</v>
       </c>
     </row>
     <row r="462" spans="1:2">
@@ -6201,7 +6219,7 @@
         <v>462</v>
       </c>
       <c r="B462" s="1">
-        <v>720</v>
+        <v>560</v>
       </c>
     </row>
     <row r="463" spans="1:2">
@@ -6209,7 +6227,7 @@
         <v>463</v>
       </c>
       <c r="B463" s="1">
-        <v>960</v>
+        <v>860</v>
       </c>
     </row>
     <row r="464" spans="1:2">
@@ -6217,7 +6235,7 @@
         <v>464</v>
       </c>
       <c r="B464" s="1">
-        <v>940</v>
+        <v>720</v>
       </c>
     </row>
     <row r="465" spans="1:2">
@@ -6225,7 +6243,7 @@
         <v>465</v>
       </c>
       <c r="B465" s="1">
-        <v>1040</v>
+        <v>960</v>
       </c>
     </row>
     <row r="466" spans="1:2">
@@ -6233,7 +6251,7 @@
         <v>466</v>
       </c>
       <c r="B466" s="1">
-        <v>920</v>
+        <v>940</v>
       </c>
     </row>
     <row r="467" spans="1:2">
@@ -6241,7 +6259,7 @@
         <v>467</v>
       </c>
       <c r="B467" s="1">
-        <v>600</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="468" spans="1:2">
@@ -6249,7 +6267,7 @@
         <v>468</v>
       </c>
       <c r="B468" s="1">
-        <v>580</v>
+        <v>920</v>
       </c>
     </row>
     <row r="469" spans="1:2">
@@ -6257,7 +6275,7 @@
         <v>469</v>
       </c>
       <c r="B469" s="1">
-        <v>820</v>
+        <v>600</v>
       </c>
     </row>
     <row r="470" spans="1:2">
@@ -6265,7 +6283,7 @@
         <v>470</v>
       </c>
       <c r="B470" s="1">
-        <v>620</v>
+        <v>580</v>
       </c>
     </row>
     <row r="471" spans="1:2">
@@ -6273,7 +6291,7 @@
         <v>471</v>
       </c>
       <c r="B471" s="1">
-        <v>900</v>
+        <v>820</v>
       </c>
     </row>
     <row r="472" spans="1:2">
@@ -6281,7 +6299,7 @@
         <v>472</v>
       </c>
       <c r="B472" s="1">
-        <v>780</v>
+        <v>620</v>
       </c>
     </row>
     <row r="473" spans="1:2">
@@ -6289,7 +6307,7 @@
         <v>473</v>
       </c>
       <c r="B473" s="1">
-        <v>700</v>
+        <v>900</v>
       </c>
     </row>
     <row r="474" spans="1:2">
@@ -6297,7 +6315,7 @@
         <v>474</v>
       </c>
       <c r="B474" s="1">
-        <v>960</v>
+        <v>780</v>
       </c>
     </row>
     <row r="475" spans="1:2">
@@ -6305,7 +6323,7 @@
         <v>475</v>
       </c>
       <c r="B475" s="1">
-        <v>600</v>
+        <v>700</v>
       </c>
     </row>
     <row r="476" spans="1:2">
@@ -6313,7 +6331,7 @@
         <v>476</v>
       </c>
       <c r="B476" s="1">
-        <v>720</v>
+        <v>960</v>
       </c>
     </row>
     <row r="477" spans="1:2">
@@ -6321,7 +6339,7 @@
         <v>477</v>
       </c>
       <c r="B477" s="1">
-        <v>780</v>
+        <v>600</v>
       </c>
     </row>
     <row r="478" spans="1:2">
@@ -6329,7 +6347,7 @@
         <v>478</v>
       </c>
       <c r="B478" s="1">
-        <v>540</v>
+        <v>720</v>
       </c>
     </row>
     <row r="479" spans="1:2">
@@ -6337,7 +6355,7 @@
         <v>479</v>
       </c>
       <c r="B479" s="1">
-        <v>720</v>
+        <v>780</v>
       </c>
     </row>
     <row r="480" spans="1:2">
@@ -6345,7 +6363,7 @@
         <v>480</v>
       </c>
       <c r="B480" s="1">
-        <v>560</v>
+        <v>540</v>
       </c>
     </row>
     <row r="481" spans="1:2">
@@ -6353,7 +6371,7 @@
         <v>481</v>
       </c>
       <c r="B481" s="1">
-        <v>740</v>
+        <v>720</v>
       </c>
     </row>
     <row r="482" spans="1:2">
@@ -6361,7 +6379,7 @@
         <v>482</v>
       </c>
       <c r="B482" s="1">
-        <v>620</v>
+        <v>560</v>
       </c>
     </row>
     <row r="483" spans="1:2">
@@ -6369,7 +6387,7 @@
         <v>483</v>
       </c>
       <c r="B483" s="1">
-        <v>860</v>
+        <v>740</v>
       </c>
     </row>
     <row r="484" spans="1:2">
@@ -6377,7 +6395,7 @@
         <v>484</v>
       </c>
       <c r="B484" s="1">
-        <v>980</v>
+        <v>620</v>
       </c>
     </row>
     <row r="485" spans="1:2">
@@ -6385,7 +6403,7 @@
         <v>485</v>
       </c>
       <c r="B485" s="1">
-        <v>740</v>
+        <v>860</v>
       </c>
     </row>
     <row r="486" spans="1:2">
@@ -6393,7 +6411,7 @@
         <v>486</v>
       </c>
       <c r="B486" s="1">
-        <v>720</v>
+        <v>980</v>
       </c>
     </row>
     <row r="487" spans="1:2">
@@ -6401,7 +6419,7 @@
         <v>487</v>
       </c>
       <c r="B487" s="1">
-        <v>920</v>
+        <v>740</v>
       </c>
     </row>
     <row r="488" spans="1:2">
@@ -6409,7 +6427,7 @@
         <v>488</v>
       </c>
       <c r="B488" s="1">
-        <v>920</v>
+        <v>720</v>
       </c>
     </row>
     <row r="489" spans="1:2">
@@ -6417,7 +6435,7 @@
         <v>489</v>
       </c>
       <c r="B489" s="1">
-        <v>720</v>
+        <v>920</v>
       </c>
     </row>
     <row r="490" spans="1:2">
@@ -6425,7 +6443,7 @@
         <v>490</v>
       </c>
       <c r="B490" s="1">
-        <v>700</v>
+        <v>920</v>
       </c>
     </row>
     <row r="491" spans="1:2">
@@ -6433,7 +6451,7 @@
         <v>491</v>
       </c>
       <c r="B491" s="1">
-        <v>840</v>
+        <v>720</v>
       </c>
     </row>
     <row r="492" spans="1:2">
@@ -6449,7 +6467,7 @@
         <v>493</v>
       </c>
       <c r="B493" s="1">
-        <v>720</v>
+        <v>840</v>
       </c>
     </row>
     <row r="494" spans="1:2">
@@ -6457,7 +6475,7 @@
         <v>494</v>
       </c>
       <c r="B494" s="1">
-        <v>800</v>
+        <v>700</v>
       </c>
     </row>
     <row r="495" spans="1:2">
@@ -6465,7 +6483,7 @@
         <v>495</v>
       </c>
       <c r="B495" s="1">
-        <v>740</v>
+        <v>720</v>
       </c>
     </row>
     <row r="496" spans="1:2">
@@ -6473,7 +6491,7 @@
         <v>496</v>
       </c>
       <c r="B496" s="1">
-        <v>720</v>
+        <v>800</v>
       </c>
     </row>
     <row r="497" spans="1:2">
@@ -6489,7 +6507,7 @@
         <v>498</v>
       </c>
       <c r="B498" s="1">
-        <v>680</v>
+        <v>720</v>
       </c>
     </row>
     <row r="499" spans="1:2">
@@ -6497,7 +6515,7 @@
         <v>499</v>
       </c>
       <c r="B499" s="1">
-        <v>720</v>
+        <v>740</v>
       </c>
     </row>
     <row r="500" spans="1:2">
@@ -6513,7 +6531,7 @@
         <v>501</v>
       </c>
       <c r="B501" s="1">
-        <v>700</v>
+        <v>720</v>
       </c>
     </row>
     <row r="502" spans="1:2">
@@ -6521,7 +6539,7 @@
         <v>502</v>
       </c>
       <c r="B502" s="1">
-        <v>820</v>
+        <v>680</v>
       </c>
     </row>
     <row r="503" spans="1:2">
@@ -6529,7 +6547,7 @@
         <v>503</v>
       </c>
       <c r="B503" s="1">
-        <v>760</v>
+        <v>700</v>
       </c>
     </row>
     <row r="504" spans="1:2">
@@ -6537,7 +6555,7 @@
         <v>504</v>
       </c>
       <c r="B504" s="1">
-        <v>720</v>
+        <v>820</v>
       </c>
     </row>
     <row r="505" spans="1:2">
@@ -6545,7 +6563,7 @@
         <v>505</v>
       </c>
       <c r="B505" s="1">
-        <v>1400</v>
+        <v>760</v>
       </c>
     </row>
     <row r="506" spans="1:2">
@@ -6561,7 +6579,7 @@
         <v>507</v>
       </c>
       <c r="B507" s="1">
-        <v>660</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="508" spans="1:2">
@@ -6569,7 +6587,7 @@
         <v>508</v>
       </c>
       <c r="B508" s="1">
-        <v>700</v>
+        <v>720</v>
       </c>
     </row>
     <row r="509" spans="1:2">
@@ -6577,7 +6595,7 @@
         <v>509</v>
       </c>
       <c r="B509" s="1">
-        <v>740</v>
+        <v>660</v>
       </c>
     </row>
     <row r="510" spans="1:2">
@@ -6585,7 +6603,7 @@
         <v>510</v>
       </c>
       <c r="B510" s="1">
-        <v>720</v>
+        <v>700</v>
       </c>
     </row>
     <row r="511" spans="1:2">
@@ -6593,7 +6611,7 @@
         <v>511</v>
       </c>
       <c r="B511" s="1">
-        <v>780</v>
+        <v>740</v>
       </c>
     </row>
     <row r="512" spans="1:2">
@@ -6601,7 +6619,7 @@
         <v>512</v>
       </c>
       <c r="B512" s="1">
-        <v>600</v>
+        <v>720</v>
       </c>
     </row>
     <row r="513" spans="1:2">
@@ -6609,7 +6627,7 @@
         <v>513</v>
       </c>
       <c r="B513" s="1">
-        <v>720</v>
+        <v>780</v>
       </c>
     </row>
     <row r="514" spans="1:2">
@@ -6617,7 +6635,7 @@
         <v>514</v>
       </c>
       <c r="B514" s="1">
-        <v>720</v>
+        <v>600</v>
       </c>
     </row>
     <row r="515" spans="1:2">
@@ -6633,7 +6651,7 @@
         <v>516</v>
       </c>
       <c r="B516" s="1">
-        <v>900</v>
+        <v>720</v>
       </c>
     </row>
     <row r="517" spans="1:2">
@@ -6641,7 +6659,7 @@
         <v>517</v>
       </c>
       <c r="B517" s="1">
-        <v>780</v>
+        <v>720</v>
       </c>
     </row>
     <row r="518" spans="1:2">
@@ -6649,7 +6667,7 @@
         <v>518</v>
       </c>
       <c r="B518" s="1">
-        <v>780</v>
+        <v>900</v>
       </c>
     </row>
     <row r="519" spans="1:2">
@@ -6657,7 +6675,7 @@
         <v>519</v>
       </c>
       <c r="B519" s="1">
-        <v>720</v>
+        <v>780</v>
       </c>
     </row>
     <row r="520" spans="1:2">
@@ -6665,7 +6683,7 @@
         <v>520</v>
       </c>
       <c r="B520" s="1">
-        <v>640</v>
+        <v>780</v>
       </c>
     </row>
     <row r="521" spans="1:2">
@@ -6673,7 +6691,7 @@
         <v>521</v>
       </c>
       <c r="B521" s="1">
-        <v>640</v>
+        <v>720</v>
       </c>
     </row>
     <row r="522" spans="1:2">
@@ -6681,7 +6699,7 @@
         <v>522</v>
       </c>
       <c r="B522" s="1">
-        <v>720</v>
+        <v>780</v>
       </c>
     </row>
     <row r="523" spans="1:2">
@@ -6689,7 +6707,7 @@
         <v>523</v>
       </c>
       <c r="B523" s="1">
-        <v>720</v>
+        <v>640</v>
       </c>
     </row>
     <row r="524" spans="1:2">
@@ -6697,7 +6715,7 @@
         <v>524</v>
       </c>
       <c r="B524" s="1">
-        <v>720</v>
+        <v>640</v>
       </c>
     </row>
     <row r="525" spans="1:2">
@@ -6705,7 +6723,7 @@
         <v>525</v>
       </c>
       <c r="B525" s="1">
-        <v>600</v>
+        <v>720</v>
       </c>
     </row>
     <row r="526" spans="1:2">
@@ -6713,7 +6731,7 @@
         <v>526</v>
       </c>
       <c r="B526" s="1">
-        <v>700</v>
+        <v>720</v>
       </c>
     </row>
     <row r="527" spans="1:2">
@@ -6721,7 +6739,7 @@
         <v>527</v>
       </c>
       <c r="B527" s="1">
-        <v>680</v>
+        <v>720</v>
       </c>
     </row>
     <row r="528" spans="1:2">
@@ -6729,7 +6747,7 @@
         <v>528</v>
       </c>
       <c r="B528" s="1">
-        <v>640</v>
+        <v>600</v>
       </c>
     </row>
     <row r="529" spans="1:2">
@@ -6737,7 +6755,7 @@
         <v>529</v>
       </c>
       <c r="B529" s="1">
-        <v>660</v>
+        <v>700</v>
       </c>
     </row>
     <row r="530" spans="1:2">
@@ -6745,7 +6763,7 @@
         <v>530</v>
       </c>
       <c r="B530" s="1">
-        <v>540</v>
+        <v>680</v>
       </c>
     </row>
     <row r="531" spans="1:2">
@@ -6753,7 +6771,7 @@
         <v>531</v>
       </c>
       <c r="B531" s="1">
-        <v>660</v>
+        <v>640</v>
       </c>
     </row>
     <row r="532" spans="1:2">
@@ -6761,7 +6779,7 @@
         <v>532</v>
       </c>
       <c r="B532" s="1">
-        <v>580</v>
+        <v>660</v>
       </c>
     </row>
     <row r="533" spans="1:2">
@@ -6769,7 +6787,7 @@
         <v>533</v>
       </c>
       <c r="B533" s="1">
-        <v>860</v>
+        <v>540</v>
       </c>
     </row>
     <row r="534" spans="1:2">
@@ -6777,7 +6795,7 @@
         <v>534</v>
       </c>
       <c r="B534" s="1">
-        <v>860</v>
+        <v>660</v>
       </c>
     </row>
     <row r="535" spans="1:2">
@@ -6785,7 +6803,7 @@
         <v>535</v>
       </c>
       <c r="B535" s="1">
-        <v>1000</v>
+        <v>580</v>
       </c>
     </row>
     <row r="536" spans="1:2">
@@ -6793,7 +6811,7 @@
         <v>536</v>
       </c>
       <c r="B536" s="1">
-        <v>900</v>
+        <v>860</v>
       </c>
     </row>
     <row r="537" spans="1:2">
@@ -6801,7 +6819,7 @@
         <v>537</v>
       </c>
       <c r="B537" s="1">
-        <v>680</v>
+        <v>860</v>
       </c>
     </row>
     <row r="538" spans="1:2">
@@ -6809,7 +6827,7 @@
         <v>538</v>
       </c>
       <c r="B538" s="1">
-        <v>1000</v>
+        <v>900</v>
       </c>
     </row>
     <row r="539" spans="1:2">
@@ -6825,7 +6843,7 @@
         <v>540</v>
       </c>
       <c r="B540" s="1">
-        <v>1020</v>
+        <v>900</v>
       </c>
     </row>
     <row r="541" spans="1:2">
@@ -6833,7 +6851,7 @@
         <v>541</v>
       </c>
       <c r="B541" s="1">
-        <v>1000</v>
+        <v>680</v>
       </c>
     </row>
     <row r="542" spans="1:2">
@@ -6841,7 +6859,7 @@
         <v>542</v>
       </c>
       <c r="B542" s="1">
-        <v>800</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="543" spans="1:2">
@@ -6849,7 +6867,7 @@
         <v>543</v>
       </c>
       <c r="B543" s="1">
-        <v>700</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="544" spans="1:2">
@@ -6857,7 +6875,7 @@
         <v>544</v>
       </c>
       <c r="B544" s="1">
-        <v>640</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="545" spans="1:2">
@@ -6865,7 +6883,7 @@
         <v>545</v>
       </c>
       <c r="B545" s="1">
-        <v>740</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="546" spans="1:2">
@@ -6873,7 +6891,7 @@
         <v>546</v>
       </c>
       <c r="B546" s="1">
-        <v>720</v>
+        <v>800</v>
       </c>
     </row>
     <row r="547" spans="1:2">
@@ -6881,7 +6899,7 @@
         <v>547</v>
       </c>
       <c r="B547" s="1">
-        <v>640</v>
+        <v>700</v>
       </c>
     </row>
     <row r="548" spans="1:2">
@@ -6889,7 +6907,7 @@
         <v>548</v>
       </c>
       <c r="B548" s="1">
-        <v>720</v>
+        <v>640</v>
       </c>
     </row>
     <row r="549" spans="1:2">
@@ -6897,7 +6915,7 @@
         <v>549</v>
       </c>
       <c r="B549" s="1">
-        <v>880</v>
+        <v>740</v>
       </c>
     </row>
     <row r="550" spans="1:2">
@@ -6905,7 +6923,7 @@
         <v>550</v>
       </c>
       <c r="B550" s="1">
-        <v>740</v>
+        <v>720</v>
       </c>
     </row>
     <row r="551" spans="1:2">
@@ -6913,7 +6931,7 @@
         <v>551</v>
       </c>
       <c r="B551" s="1">
-        <v>600</v>
+        <v>640</v>
       </c>
     </row>
     <row r="552" spans="1:2">
@@ -6921,7 +6939,7 @@
         <v>552</v>
       </c>
       <c r="B552" s="1">
-        <v>820</v>
+        <v>720</v>
       </c>
     </row>
     <row r="553" spans="1:2">
@@ -6929,7 +6947,7 @@
         <v>553</v>
       </c>
       <c r="B553" s="1">
-        <v>600</v>
+        <v>880</v>
       </c>
     </row>
     <row r="554" spans="1:2">
@@ -6937,7 +6955,7 @@
         <v>554</v>
       </c>
       <c r="B554" s="1">
-        <v>640</v>
+        <v>740</v>
       </c>
     </row>
     <row r="555" spans="1:2">
@@ -6945,7 +6963,7 @@
         <v>555</v>
       </c>
       <c r="B555" s="1">
-        <v>740</v>
+        <v>600</v>
       </c>
     </row>
     <row r="556" spans="1:2">
@@ -6953,7 +6971,7 @@
         <v>556</v>
       </c>
       <c r="B556" s="1">
-        <v>900</v>
+        <v>820</v>
       </c>
     </row>
     <row r="557" spans="1:2">
@@ -6961,7 +6979,7 @@
         <v>557</v>
       </c>
       <c r="B557" s="1">
-        <v>900</v>
+        <v>600</v>
       </c>
     </row>
     <row r="558" spans="1:2">
@@ -6969,7 +6987,7 @@
         <v>558</v>
       </c>
       <c r="B558" s="1">
-        <v>720</v>
+        <v>640</v>
       </c>
     </row>
     <row r="559" spans="1:2">
@@ -6977,7 +6995,7 @@
         <v>559</v>
       </c>
       <c r="B559" s="1">
-        <v>960</v>
+        <v>780</v>
       </c>
     </row>
     <row r="560" spans="1:2">
@@ -6985,7 +7003,7 @@
         <v>560</v>
       </c>
       <c r="B560" s="1">
-        <v>1020</v>
+        <v>900</v>
       </c>
     </row>
     <row r="561" spans="1:2">
@@ -6993,7 +7011,7 @@
         <v>561</v>
       </c>
       <c r="B561" s="1">
-        <v>780</v>
+        <v>900</v>
       </c>
     </row>
     <row r="562" spans="1:2">
@@ -7001,7 +7019,7 @@
         <v>562</v>
       </c>
       <c r="B562" s="1">
-        <v>700</v>
+        <v>720</v>
       </c>
     </row>
     <row r="563" spans="1:2">
@@ -7009,7 +7027,7 @@
         <v>563</v>
       </c>
       <c r="B563" s="1">
-        <v>640</v>
+        <v>960</v>
       </c>
     </row>
     <row r="564" spans="1:2">
@@ -7017,7 +7035,7 @@
         <v>564</v>
       </c>
       <c r="B564" s="1">
-        <v>780</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="565" spans="1:2">
@@ -7025,7 +7043,7 @@
         <v>565</v>
       </c>
       <c r="B565" s="1">
-        <v>1020</v>
+        <v>780</v>
       </c>
     </row>
     <row r="566" spans="1:2">
@@ -7033,7 +7051,7 @@
         <v>566</v>
       </c>
       <c r="B566" s="1">
-        <v>780</v>
+        <v>700</v>
       </c>
     </row>
     <row r="567" spans="1:2">
@@ -7041,7 +7059,7 @@
         <v>567</v>
       </c>
       <c r="B567" s="1">
-        <v>1000</v>
+        <v>640</v>
       </c>
     </row>
     <row r="568" spans="1:2">
@@ -7049,7 +7067,7 @@
         <v>568</v>
       </c>
       <c r="B568" s="1">
-        <v>1000</v>
+        <v>780</v>
       </c>
     </row>
     <row r="569" spans="1:2">
@@ -7057,7 +7075,7 @@
         <v>569</v>
       </c>
       <c r="B569" s="1">
-        <v>780</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="570" spans="1:2">
@@ -7065,7 +7083,7 @@
         <v>570</v>
       </c>
       <c r="B570" s="1">
-        <v>720</v>
+        <v>780</v>
       </c>
     </row>
     <row r="571" spans="1:2">
@@ -7073,7 +7091,7 @@
         <v>571</v>
       </c>
       <c r="B571" s="1">
-        <v>680</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="572" spans="1:2">
@@ -7081,7 +7099,7 @@
         <v>572</v>
       </c>
       <c r="B572" s="1">
-        <v>700</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="573" spans="1:2">
@@ -7089,7 +7107,7 @@
         <v>573</v>
       </c>
       <c r="B573" s="1">
-        <v>680</v>
+        <v>780</v>
       </c>
     </row>
     <row r="574" spans="1:2">
@@ -7097,7 +7115,7 @@
         <v>574</v>
       </c>
       <c r="B574" s="1">
-        <v>740</v>
+        <v>720</v>
       </c>
     </row>
     <row r="575" spans="1:2">
@@ -7113,7 +7131,7 @@
         <v>576</v>
       </c>
       <c r="B576" s="1">
-        <v>1000</v>
+        <v>700</v>
       </c>
     </row>
     <row r="577" spans="1:2">
@@ -7121,7 +7139,7 @@
         <v>577</v>
       </c>
       <c r="B577" s="1">
-        <v>920</v>
+        <v>680</v>
       </c>
     </row>
     <row r="578" spans="1:2">
@@ -7129,7 +7147,7 @@
         <v>578</v>
       </c>
       <c r="B578" s="1">
-        <v>860</v>
+        <v>740</v>
       </c>
     </row>
     <row r="579" spans="1:2">
@@ -7137,7 +7155,7 @@
         <v>579</v>
       </c>
       <c r="B579" s="1">
-        <v>740</v>
+        <v>680</v>
       </c>
     </row>
     <row r="580" spans="1:2">
@@ -7145,7 +7163,7 @@
         <v>580</v>
       </c>
       <c r="B580" s="1">
-        <v>900</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="581" spans="1:2">
@@ -7153,7 +7171,7 @@
         <v>581</v>
       </c>
       <c r="B581" s="1">
-        <v>740</v>
+        <v>920</v>
       </c>
     </row>
     <row r="582" spans="1:2">
@@ -7161,7 +7179,7 @@
         <v>582</v>
       </c>
       <c r="B582" s="1">
-        <v>840</v>
+        <v>860</v>
       </c>
     </row>
     <row r="583" spans="1:2">
@@ -7169,7 +7187,7 @@
         <v>583</v>
       </c>
       <c r="B583" s="1">
-        <v>720</v>
+        <v>740</v>
       </c>
     </row>
     <row r="584" spans="1:2">
@@ -7177,7 +7195,7 @@
         <v>584</v>
       </c>
       <c r="B584" s="1">
-        <v>820</v>
+        <v>900</v>
       </c>
     </row>
     <row r="585" spans="1:2">
@@ -7185,7 +7203,7 @@
         <v>585</v>
       </c>
       <c r="B585" s="1">
-        <v>1000</v>
+        <v>740</v>
       </c>
     </row>
     <row r="586" spans="1:2">
@@ -7193,7 +7211,7 @@
         <v>586</v>
       </c>
       <c r="B586" s="1">
-        <v>900</v>
+        <v>840</v>
       </c>
     </row>
     <row r="587" spans="1:2">
@@ -7201,7 +7219,7 @@
         <v>587</v>
       </c>
       <c r="B587" s="1">
-        <v>900</v>
+        <v>720</v>
       </c>
     </row>
     <row r="588" spans="1:2">
@@ -7209,7 +7227,7 @@
         <v>588</v>
       </c>
       <c r="B588" s="1">
-        <v>1000</v>
+        <v>820</v>
       </c>
     </row>
     <row r="589" spans="1:2">
@@ -7217,7 +7235,7 @@
         <v>589</v>
       </c>
       <c r="B589" s="1">
-        <v>780</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="590" spans="1:2">
@@ -7225,7 +7243,7 @@
         <v>590</v>
       </c>
       <c r="B590" s="1">
-        <v>880</v>
+        <v>900</v>
       </c>
     </row>
     <row r="591" spans="1:2">
@@ -7233,7 +7251,7 @@
         <v>591</v>
       </c>
       <c r="B591" s="1">
-        <v>780</v>
+        <v>900</v>
       </c>
     </row>
     <row r="592" spans="1:2">
@@ -7241,7 +7259,7 @@
         <v>592</v>
       </c>
       <c r="B592" s="1">
-        <v>740</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="593" spans="1:2">
@@ -7249,7 +7267,7 @@
         <v>593</v>
       </c>
       <c r="B593" s="1">
-        <v>900</v>
+        <v>780</v>
       </c>
     </row>
     <row r="594" spans="1:2">
@@ -7257,7 +7275,7 @@
         <v>594</v>
       </c>
       <c r="B594" s="1">
-        <v>660</v>
+        <v>880</v>
       </c>
     </row>
     <row r="595" spans="1:2">
@@ -7265,7 +7283,7 @@
         <v>595</v>
       </c>
       <c r="B595" s="1">
-        <v>700</v>
+        <v>780</v>
       </c>
     </row>
     <row r="596" spans="1:2">
@@ -7273,7 +7291,7 @@
         <v>596</v>
       </c>
       <c r="B596" s="1">
-        <v>680</v>
+        <v>740</v>
       </c>
     </row>
     <row r="597" spans="1:2">
@@ -7281,7 +7299,7 @@
         <v>597</v>
       </c>
       <c r="B597" s="1">
-        <v>660</v>
+        <v>900</v>
       </c>
     </row>
     <row r="598" spans="1:2">
@@ -7289,7 +7307,7 @@
         <v>598</v>
       </c>
       <c r="B598" s="1">
-        <v>440</v>
+        <v>660</v>
       </c>
     </row>
     <row r="599" spans="1:2">
@@ -7305,7 +7323,7 @@
         <v>600</v>
       </c>
       <c r="B600" s="1">
-        <v>800</v>
+        <v>680</v>
       </c>
     </row>
     <row r="601" spans="1:2">
@@ -7313,7 +7331,7 @@
         <v>601</v>
       </c>
       <c r="B601" s="1">
-        <v>720</v>
+        <v>660</v>
       </c>
     </row>
     <row r="602" spans="1:2">
@@ -7321,7 +7339,7 @@
         <v>602</v>
       </c>
       <c r="B602" s="1">
-        <v>600</v>
+        <v>440</v>
       </c>
     </row>
     <row r="603" spans="1:2">
@@ -7329,7 +7347,7 @@
         <v>603</v>
       </c>
       <c r="B603" s="1">
-        <v>560</v>
+        <v>700</v>
       </c>
     </row>
     <row r="604" spans="1:2">
@@ -7337,7 +7355,7 @@
         <v>604</v>
       </c>
       <c r="B604" s="1">
-        <v>900</v>
+        <v>800</v>
       </c>
     </row>
     <row r="605" spans="1:2">
@@ -7345,7 +7363,7 @@
         <v>605</v>
       </c>
       <c r="B605" s="1">
-        <v>800</v>
+        <v>720</v>
       </c>
     </row>
     <row r="606" spans="1:2">
@@ -7353,7 +7371,7 @@
         <v>606</v>
       </c>
       <c r="B606" s="1">
-        <v>780</v>
+        <v>600</v>
       </c>
     </row>
     <row r="607" spans="1:2">
@@ -7361,7 +7379,7 @@
         <v>607</v>
       </c>
       <c r="B607" s="1">
-        <v>920</v>
+        <v>560</v>
       </c>
     </row>
     <row r="608" spans="1:2">
@@ -7369,7 +7387,7 @@
         <v>608</v>
       </c>
       <c r="B608" s="1">
-        <v>740</v>
+        <v>900</v>
       </c>
     </row>
     <row r="609" spans="1:2">
@@ -7377,7 +7395,7 @@
         <v>609</v>
       </c>
       <c r="B609" s="1">
-        <v>940</v>
+        <v>800</v>
       </c>
     </row>
     <row r="610" spans="1:2">
@@ -7385,7 +7403,7 @@
         <v>610</v>
       </c>
       <c r="B610" s="1">
-        <v>980</v>
+        <v>780</v>
       </c>
     </row>
     <row r="611" spans="1:2">
@@ -7401,7 +7419,7 @@
         <v>612</v>
       </c>
       <c r="B612" s="1">
-        <v>780</v>
+        <v>740</v>
       </c>
     </row>
     <row r="613" spans="1:2">
@@ -7409,7 +7427,7 @@
         <v>613</v>
       </c>
       <c r="B613" s="1">
-        <v>860</v>
+        <v>940</v>
       </c>
     </row>
     <row r="614" spans="1:2">
@@ -7417,7 +7435,7 @@
         <v>614</v>
       </c>
       <c r="B614" s="1">
-        <v>920</v>
+        <v>980</v>
       </c>
     </row>
     <row r="615" spans="1:2">
@@ -7425,7 +7443,7 @@
         <v>615</v>
       </c>
       <c r="B615" s="1">
-        <v>680</v>
+        <v>920</v>
       </c>
     </row>
     <row r="616" spans="1:2">
@@ -7433,7 +7451,7 @@
         <v>616</v>
       </c>
       <c r="B616" s="1">
-        <v>820</v>
+        <v>780</v>
       </c>
     </row>
     <row r="617" spans="1:2">
@@ -7441,7 +7459,7 @@
         <v>617</v>
       </c>
       <c r="B617" s="1">
-        <v>960</v>
+        <v>860</v>
       </c>
     </row>
     <row r="618" spans="1:2">
@@ -7449,7 +7467,7 @@
         <v>618</v>
       </c>
       <c r="B618" s="1">
-        <v>740</v>
+        <v>920</v>
       </c>
     </row>
     <row r="619" spans="1:2">
@@ -7457,7 +7475,7 @@
         <v>619</v>
       </c>
       <c r="B619" s="1">
-        <v>1000</v>
+        <v>680</v>
       </c>
     </row>
     <row r="620" spans="1:2">
@@ -7465,7 +7483,7 @@
         <v>620</v>
       </c>
       <c r="B620" s="1">
-        <v>860</v>
+        <v>820</v>
       </c>
     </row>
     <row r="621" spans="1:2">
@@ -7473,7 +7491,7 @@
         <v>621</v>
       </c>
       <c r="B621" s="1">
-        <v>780</v>
+        <v>960</v>
       </c>
     </row>
     <row r="622" spans="1:2">
@@ -7481,7 +7499,7 @@
         <v>622</v>
       </c>
       <c r="B622" s="1">
-        <v>660</v>
+        <v>740</v>
       </c>
     </row>
     <row r="623" spans="1:2">
@@ -7489,7 +7507,7 @@
         <v>623</v>
       </c>
       <c r="B623" s="1">
-        <v>840</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="624" spans="1:2">
@@ -7497,7 +7515,7 @@
         <v>624</v>
       </c>
       <c r="B624" s="1">
-        <v>780</v>
+        <v>860</v>
       </c>
     </row>
     <row r="625" spans="1:2">
@@ -7505,7 +7523,7 @@
         <v>625</v>
       </c>
       <c r="B625" s="1">
-        <v>820</v>
+        <v>780</v>
       </c>
     </row>
     <row r="626" spans="1:2">
@@ -7513,7 +7531,7 @@
         <v>626</v>
       </c>
       <c r="B626" s="1">
-        <v>760</v>
+        <v>660</v>
       </c>
     </row>
     <row r="627" spans="1:2">
@@ -7521,7 +7539,7 @@
         <v>627</v>
       </c>
       <c r="B627" s="1">
-        <v>740</v>
+        <v>840</v>
       </c>
     </row>
     <row r="628" spans="1:2">
@@ -7537,7 +7555,7 @@
         <v>629</v>
       </c>
       <c r="B629" s="1">
-        <v>600</v>
+        <v>820</v>
       </c>
     </row>
     <row r="630" spans="1:2">
@@ -7545,7 +7563,7 @@
         <v>630</v>
       </c>
       <c r="B630" s="1">
-        <v>840</v>
+        <v>760</v>
       </c>
     </row>
     <row r="631" spans="1:2">
@@ -7553,7 +7571,7 @@
         <v>631</v>
       </c>
       <c r="B631" s="1">
-        <v>660</v>
+        <v>740</v>
       </c>
     </row>
     <row r="632" spans="1:2">
@@ -7561,7 +7579,7 @@
         <v>632</v>
       </c>
       <c r="B632" s="1">
-        <v>740</v>
+        <v>780</v>
       </c>
     </row>
     <row r="633" spans="1:2">
@@ -7569,7 +7587,7 @@
         <v>633</v>
       </c>
       <c r="B633" s="1">
-        <v>760</v>
+        <v>600</v>
       </c>
     </row>
     <row r="634" spans="1:2">
@@ -7577,7 +7595,7 @@
         <v>634</v>
       </c>
       <c r="B634" s="1">
-        <v>700</v>
+        <v>840</v>
       </c>
     </row>
     <row r="635" spans="1:2">
@@ -7585,7 +7603,7 @@
         <v>635</v>
       </c>
       <c r="B635" s="1">
-        <v>860</v>
+        <v>660</v>
       </c>
     </row>
     <row r="636" spans="1:2">
@@ -7593,7 +7611,7 @@
         <v>636</v>
       </c>
       <c r="B636" s="1">
-        <v>680</v>
+        <v>740</v>
       </c>
     </row>
     <row r="637" spans="1:2">
@@ -7601,7 +7619,7 @@
         <v>637</v>
       </c>
       <c r="B637" s="1">
-        <v>740</v>
+        <v>760</v>
       </c>
     </row>
     <row r="638" spans="1:2">
@@ -7609,7 +7627,7 @@
         <v>638</v>
       </c>
       <c r="B638" s="1">
-        <v>720</v>
+        <v>700</v>
       </c>
     </row>
     <row r="639" spans="1:2">
@@ -7617,7 +7635,7 @@
         <v>639</v>
       </c>
       <c r="B639" s="1">
-        <v>720</v>
+        <v>860</v>
       </c>
     </row>
     <row r="640" spans="1:2">
@@ -7625,7 +7643,7 @@
         <v>640</v>
       </c>
       <c r="B640" s="1">
-        <v>600</v>
+        <v>680</v>
       </c>
     </row>
     <row r="641" spans="1:2">
@@ -7633,7 +7651,7 @@
         <v>641</v>
       </c>
       <c r="B641" s="1">
-        <v>600</v>
+        <v>740</v>
       </c>
     </row>
     <row r="642" spans="1:2">
@@ -7641,7 +7659,7 @@
         <v>642</v>
       </c>
       <c r="B642" s="1">
-        <v>500</v>
+        <v>780</v>
       </c>
     </row>
     <row r="643" spans="1:2">
@@ -7649,7 +7667,7 @@
         <v>643</v>
       </c>
       <c r="B643" s="1">
-        <v>600</v>
+        <v>720</v>
       </c>
     </row>
     <row r="644" spans="1:2">
@@ -7657,7 +7675,7 @@
         <v>644</v>
       </c>
       <c r="B644" s="1">
-        <v>920</v>
+        <v>720</v>
       </c>
     </row>
     <row r="645" spans="1:2">
@@ -7665,7 +7683,7 @@
         <v>645</v>
       </c>
       <c r="B645" s="1">
-        <v>1000</v>
+        <v>600</v>
       </c>
     </row>
     <row r="646" spans="1:2">
@@ -7673,7 +7691,7 @@
         <v>646</v>
       </c>
       <c r="B646" s="1">
-        <v>1040</v>
+        <v>600</v>
       </c>
     </row>
     <row r="647" spans="1:2">
@@ -7681,7 +7699,7 @@
         <v>647</v>
       </c>
       <c r="B647" s="1">
-        <v>940</v>
+        <v>500</v>
       </c>
     </row>
     <row r="648" spans="1:2">
@@ -7689,7 +7707,7 @@
         <v>648</v>
       </c>
       <c r="B648" s="1">
-        <v>900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="649" spans="1:2">
@@ -7697,7 +7715,7 @@
         <v>649</v>
       </c>
       <c r="B649" s="1">
-        <v>1000</v>
+        <v>920</v>
       </c>
     </row>
     <row r="650" spans="1:2">
@@ -7705,7 +7723,7 @@
         <v>650</v>
       </c>
       <c r="B650" s="1">
-        <v>740</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="651" spans="1:2">
@@ -7713,7 +7731,7 @@
         <v>651</v>
       </c>
       <c r="B651" s="1">
-        <v>440</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="652" spans="1:2">
@@ -7721,7 +7739,7 @@
         <v>652</v>
       </c>
       <c r="B652" s="1">
-        <v>500</v>
+        <v>940</v>
       </c>
     </row>
     <row r="653" spans="1:2">
@@ -7729,7 +7747,7 @@
         <v>653</v>
       </c>
       <c r="B653" s="1">
-        <v>440</v>
+        <v>900</v>
       </c>
     </row>
     <row r="654" spans="1:2">
@@ -7737,7 +7755,7 @@
         <v>654</v>
       </c>
       <c r="B654" s="1">
-        <v>560</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="655" spans="1:2">
@@ -7745,7 +7763,7 @@
         <v>655</v>
       </c>
       <c r="B655" s="1">
-        <v>500</v>
+        <v>740</v>
       </c>
     </row>
     <row r="656" spans="1:2">
@@ -7753,7 +7771,7 @@
         <v>656</v>
       </c>
       <c r="B656" s="1">
-        <v>740</v>
+        <v>440</v>
       </c>
     </row>
     <row r="657" spans="1:2">
@@ -7761,7 +7779,7 @@
         <v>657</v>
       </c>
       <c r="B657" s="1">
-        <v>760</v>
+        <v>500</v>
       </c>
     </row>
     <row r="658" spans="1:2">
@@ -7769,7 +7787,7 @@
         <v>658</v>
       </c>
       <c r="B658" s="1">
-        <v>760</v>
+        <v>440</v>
       </c>
     </row>
     <row r="659" spans="1:2">
@@ -7777,7 +7795,7 @@
         <v>659</v>
       </c>
       <c r="B659" s="1">
-        <v>400</v>
+        <v>560</v>
       </c>
     </row>
     <row r="660" spans="1:2">
@@ -7785,7 +7803,7 @@
         <v>660</v>
       </c>
       <c r="B660" s="1">
-        <v>400</v>
+        <v>500</v>
       </c>
     </row>
     <row r="661" spans="1:2">
@@ -7793,7 +7811,7 @@
         <v>661</v>
       </c>
       <c r="B661" s="1">
-        <v>380</v>
+        <v>740</v>
       </c>
     </row>
     <row r="662" spans="1:2">
@@ -7801,7 +7819,7 @@
         <v>662</v>
       </c>
       <c r="B662" s="1">
-        <v>380</v>
+        <v>760</v>
       </c>
     </row>
     <row r="663" spans="1:2">
@@ -7809,7 +7827,7 @@
         <v>663</v>
       </c>
       <c r="B663" s="1">
-        <v>380</v>
+        <v>760</v>
       </c>
     </row>
     <row r="664" spans="1:2">
@@ -7817,7 +7835,7 @@
         <v>664</v>
       </c>
       <c r="B664" s="1">
-        <v>520</v>
+        <v>400</v>
       </c>
     </row>
     <row r="665" spans="1:2">
@@ -7825,7 +7843,7 @@
         <v>665</v>
       </c>
       <c r="B665" s="1">
-        <v>700</v>
+        <v>400</v>
       </c>
     </row>
     <row r="666" spans="1:2">
@@ -7833,7 +7851,7 @@
         <v>666</v>
       </c>
       <c r="B666" s="1">
-        <v>860</v>
+        <v>380</v>
       </c>
     </row>
     <row r="667" spans="1:2">
@@ -7841,7 +7859,7 @@
         <v>667</v>
       </c>
       <c r="B667" s="1">
-        <v>680</v>
+        <v>380</v>
       </c>
     </row>
     <row r="668" spans="1:2">
@@ -7849,7 +7867,7 @@
         <v>668</v>
       </c>
       <c r="B668" s="1">
-        <v>740</v>
+        <v>380</v>
       </c>
     </row>
     <row r="669" spans="1:2">
@@ -7857,7 +7875,7 @@
         <v>669</v>
       </c>
       <c r="B669" s="1">
-        <v>720</v>
+        <v>520</v>
       </c>
     </row>
     <row r="670" spans="1:2">
@@ -7865,7 +7883,7 @@
         <v>670</v>
       </c>
       <c r="B670" s="1">
-        <v>720</v>
+        <v>700</v>
       </c>
     </row>
     <row r="671" spans="1:2">
@@ -7873,7 +7891,7 @@
         <v>671</v>
       </c>
       <c r="B671" s="1">
-        <v>600</v>
+        <v>860</v>
       </c>
     </row>
     <row r="672" spans="1:2">
@@ -7881,7 +7899,7 @@
         <v>672</v>
       </c>
       <c r="B672" s="1">
-        <v>600</v>
+        <v>680</v>
       </c>
     </row>
     <row r="673" spans="1:2">
@@ -7889,7 +7907,7 @@
         <v>673</v>
       </c>
       <c r="B673" s="1">
-        <v>500</v>
+        <v>740</v>
       </c>
     </row>
     <row r="674" spans="1:2">
@@ -7897,7 +7915,7 @@
         <v>674</v>
       </c>
       <c r="B674" s="1">
-        <v>600</v>
+        <v>780</v>
       </c>
     </row>
     <row r="675" spans="1:2">
@@ -7905,7 +7923,7 @@
         <v>675</v>
       </c>
       <c r="B675" s="1">
-        <v>840</v>
+        <v>720</v>
       </c>
     </row>
     <row r="676" spans="1:2">
@@ -7913,7 +7931,7 @@
         <v>676</v>
       </c>
       <c r="B676" s="1">
-        <v>900</v>
+        <v>720</v>
       </c>
     </row>
     <row r="677" spans="1:2">
@@ -7921,7 +7939,7 @@
         <v>677</v>
       </c>
       <c r="B677" s="1">
-        <v>900</v>
+        <v>600</v>
       </c>
     </row>
     <row r="678" spans="1:2">
@@ -7929,7 +7947,7 @@
         <v>678</v>
       </c>
       <c r="B678" s="1">
-        <v>920</v>
+        <v>600</v>
       </c>
     </row>
     <row r="679" spans="1:2">
@@ -7937,7 +7955,7 @@
         <v>679</v>
       </c>
       <c r="B679" s="1">
-        <v>1000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="680" spans="1:2">
@@ -7945,7 +7963,7 @@
         <v>680</v>
       </c>
       <c r="B680" s="1">
-        <v>1040</v>
+        <v>760</v>
       </c>
     </row>
     <row r="681" spans="1:2">
@@ -7953,7 +7971,7 @@
         <v>681</v>
       </c>
       <c r="B681" s="1">
-        <v>940</v>
+        <v>840</v>
       </c>
     </row>
     <row r="682" spans="1:2">
@@ -7969,7 +7987,7 @@
         <v>683</v>
       </c>
       <c r="B683" s="1">
-        <v>1000</v>
+        <v>900</v>
       </c>
     </row>
     <row r="684" spans="1:2">
@@ -7977,7 +7995,7 @@
         <v>684</v>
       </c>
       <c r="B684" s="1">
-        <v>740</v>
+        <v>920</v>
       </c>
     </row>
     <row r="685" spans="1:2">
@@ -7985,7 +8003,7 @@
         <v>685</v>
       </c>
       <c r="B685" s="1">
-        <v>440</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="686" spans="1:2">
@@ -7993,7 +8011,7 @@
         <v>686</v>
       </c>
       <c r="B686" s="1">
-        <v>500</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="687" spans="1:2">
@@ -8001,7 +8019,7 @@
         <v>687</v>
       </c>
       <c r="B687" s="1">
-        <v>440</v>
+        <v>940</v>
       </c>
     </row>
     <row r="688" spans="1:2">
@@ -8009,7 +8027,7 @@
         <v>688</v>
       </c>
       <c r="B688" s="1">
-        <v>560</v>
+        <v>900</v>
       </c>
     </row>
     <row r="689" spans="1:2">
@@ -8017,7 +8035,7 @@
         <v>689</v>
       </c>
       <c r="B689" s="1">
-        <v>500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="690" spans="1:2">
@@ -8033,7 +8051,7 @@
         <v>691</v>
       </c>
       <c r="B691" s="1">
-        <v>380</v>
+        <v>440</v>
       </c>
     </row>
     <row r="692" spans="1:2">
@@ -8041,7 +8059,7 @@
         <v>692</v>
       </c>
       <c r="B692" s="1">
-        <v>380</v>
+        <v>500</v>
       </c>
     </row>
     <row r="693" spans="1:2">
@@ -8049,7 +8067,7 @@
         <v>693</v>
       </c>
       <c r="B693" s="1">
-        <v>380</v>
+        <v>440</v>
       </c>
     </row>
     <row r="694" spans="1:2">
@@ -8057,7 +8075,7 @@
         <v>694</v>
       </c>
       <c r="B694" s="1">
-        <v>480</v>
+        <v>560</v>
       </c>
     </row>
     <row r="695" spans="1:2">
@@ -8065,7 +8083,7 @@
         <v>695</v>
       </c>
       <c r="B695" s="1">
-        <v>480</v>
+        <v>500</v>
       </c>
     </row>
     <row r="696" spans="1:2">
@@ -8073,7 +8091,7 @@
         <v>696</v>
       </c>
       <c r="B696" s="1">
-        <v>480</v>
+        <v>740</v>
       </c>
     </row>
     <row r="697" spans="1:2">
@@ -8081,7 +8099,7 @@
         <v>697</v>
       </c>
       <c r="B697" s="1">
-        <v>520</v>
+        <v>380</v>
       </c>
     </row>
     <row r="698" spans="1:2">
@@ -8089,7 +8107,7 @@
         <v>698</v>
       </c>
       <c r="B698" s="1">
-        <v>520</v>
+        <v>380</v>
       </c>
     </row>
     <row r="699" spans="1:2">
@@ -8097,7 +8115,7 @@
         <v>699</v>
       </c>
       <c r="B699" s="1">
-        <v>440</v>
+        <v>380</v>
       </c>
     </row>
     <row r="700" spans="1:2">
@@ -8105,7 +8123,7 @@
         <v>700</v>
       </c>
       <c r="B700" s="1">
-        <v>420</v>
+        <v>480</v>
       </c>
     </row>
     <row r="701" spans="1:2">
@@ -8113,7 +8131,7 @@
         <v>701</v>
       </c>
       <c r="B701" s="1">
-        <v>380</v>
+        <v>480</v>
       </c>
     </row>
     <row r="702" spans="1:2">
@@ -8121,7 +8139,7 @@
         <v>702</v>
       </c>
       <c r="B702" s="1">
-        <v>600</v>
+        <v>480</v>
       </c>
     </row>
     <row r="703" spans="1:2">
@@ -8129,7 +8147,7 @@
         <v>703</v>
       </c>
       <c r="B703" s="1">
-        <v>760</v>
+        <v>520</v>
       </c>
     </row>
     <row r="704" spans="1:2">
@@ -8137,7 +8155,7 @@
         <v>704</v>
       </c>
       <c r="B704" s="1">
-        <v>600</v>
+        <v>520</v>
       </c>
     </row>
     <row r="705" spans="1:2">
@@ -8145,7 +8163,7 @@
         <v>705</v>
       </c>
       <c r="B705" s="1">
-        <v>580</v>
+        <v>440</v>
       </c>
     </row>
     <row r="706" spans="1:2">
@@ -8153,7 +8171,7 @@
         <v>706</v>
       </c>
       <c r="B706" s="1">
-        <v>560</v>
+        <v>420</v>
       </c>
     </row>
     <row r="707" spans="1:2">
@@ -8161,7 +8179,7 @@
         <v>707</v>
       </c>
       <c r="B707" s="1">
-        <v>580</v>
+        <v>380</v>
       </c>
     </row>
     <row r="708" spans="1:2">
@@ -8169,7 +8187,7 @@
         <v>708</v>
       </c>
       <c r="B708" s="1">
-        <v>620</v>
+        <v>600</v>
       </c>
     </row>
     <row r="709" spans="1:2">
@@ -8177,7 +8195,7 @@
         <v>709</v>
       </c>
       <c r="B709" s="1">
-        <v>560</v>
+        <v>760</v>
       </c>
     </row>
     <row r="710" spans="1:2">
@@ -8185,6 +8203,54 @@
         <v>710</v>
       </c>
       <c r="B710" s="1">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="711" spans="1:2">
+      <c r="A711" s="1" t="s">
+        <v>711</v>
+      </c>
+      <c r="B711" s="1">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="712" spans="1:2">
+      <c r="A712" s="1" t="s">
+        <v>712</v>
+      </c>
+      <c r="B712" s="1">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="713" spans="1:2">
+      <c r="A713" s="1" t="s">
+        <v>713</v>
+      </c>
+      <c r="B713" s="1">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="714" spans="1:2">
+      <c r="A714" s="1" t="s">
+        <v>714</v>
+      </c>
+      <c r="B714" s="1">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="715" spans="1:2">
+      <c r="A715" s="1" t="s">
+        <v>715</v>
+      </c>
+      <c r="B715" s="1">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="716" spans="1:2">
+      <c r="A716" s="1" t="s">
+        <v>716</v>
+      </c>
+      <c r="B716" s="1">
         <v>560</v>
       </c>
     </row>

</xml_diff>